<commit_message>
#110 eSpark BOM for 5 Boards Updated PCBWay and LCSC BOM remaining
</commit_message>
<xml_diff>
--- a/Deliverables/BOM/eSpark-BOM-v2.1.xlsx
+++ b/Deliverables/BOM/eSpark-BOM-v2.1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\Melih-SoundSensor\Deliverables\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07670EB1-03E7-4C59-8C4B-9D4D8AC67800}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10616AFF-8CD5-4EE6-9A27-304F451BBA3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1788" uniqueCount="285">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1778" uniqueCount="296">
   <si>
     <t>Component list</t>
   </si>
@@ -892,6 +892,39 @@
   </si>
   <si>
     <t>RS-03K104JT</t>
+  </si>
+  <si>
+    <t>C3, C5, C7, C9, C11, C13, C15, C17, C24, C25, C27, C29, C30, C32, C35, C39, C42, C53, C55, C64, C65, C66, C67, C70, C72, C76, C78, C85, C90, C91, C92, C93, C94, C95, C98, C99, C108, C112, C113, C114, C116, C118, C120, C128, C135, C136, C165, C166, C167, C168, C#2</t>
+  </si>
+  <si>
+    <t>C45, C46, C47, C48, C49, C50, C51, C52, C97, C100, C101, C102, C103, C104, C105, C106, C107, C119, C122, C123, C126, C130, C133, C134, C141, C142, C143, C144, C145, C146, C147, C148, C149, C150, C151, C152, C153, C154, C155, C156, C157, C158, C159, C160, C161, C162, C163, C164</t>
+  </si>
+  <si>
+    <t>C2168289</t>
+  </si>
+  <si>
+    <t>Ferrite Bead</t>
+  </si>
+  <si>
+    <t>FB1, FB2</t>
+  </si>
+  <si>
+    <t>FERRITE BEAD 120 OHM 0603 1LN</t>
+  </si>
+  <si>
+    <t>IND-0603 (1608 Metric)</t>
+  </si>
+  <si>
+    <t>BLM18SG121TN1D</t>
+  </si>
+  <si>
+    <t>Murata</t>
+  </si>
+  <si>
+    <t>C113030</t>
+  </si>
+  <si>
+    <t>C1,C2, C23, C26, C28, C137, C138, C139, C140</t>
   </si>
 </sst>
 </file>
@@ -1407,7 +1440,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="109">
+  <cellXfs count="114">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1713,6 +1746,21 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2218,7 +2266,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C605574B-18B4-4F8A-BF86-58CC88FF11BE}">
-  <dimension ref="A1:S52"/>
+  <dimension ref="A1:S51"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3" bestFit="1" customWidth="1"/>
@@ -2482,7 +2530,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="10" spans="1:19" s="64" customFormat="1" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:19" s="64" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="63"/>
       <c r="B10" s="37">
         <f>ROW(B10) - ROW($B$9)</f>
@@ -2492,7 +2540,7 @@
         <v>7</v>
       </c>
       <c r="D10" s="71" t="s">
-        <v>13</v>
+        <v>295</v>
       </c>
       <c r="E10" s="67" t="s">
         <v>51</v>
@@ -2516,14 +2564,14 @@
         <v>181</v>
       </c>
       <c r="L10" s="61">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="M10" s="61">
         <f>L10*5</f>
-        <v>100</v>
+        <v>45</v>
       </c>
       <c r="N10" s="61">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="O10" s="69" t="s">
         <v>223</v>
@@ -2533,87 +2581,87 @@
       </c>
       <c r="Q10" s="70">
         <f>P10*N10</f>
-        <v>2.8319999999999999</v>
+        <v>1.4159999999999999</v>
       </c>
       <c r="R10" s="67"/>
       <c r="S10" s="70"/>
     </row>
-    <row r="11" spans="1:19" s="64" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:19" s="64" customFormat="1" ht="84.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="63"/>
       <c r="B11" s="37">
-        <f t="shared" ref="B11:B49" si="0">ROW(B11) - ROW($B$9)</f>
+        <f>ROW(B11) - ROW($B$9)</f>
         <v>2</v>
       </c>
-      <c r="C11" s="52" t="s">
+      <c r="C11" s="53" t="s">
         <v>7</v>
       </c>
-      <c r="D11" s="72" t="s">
-        <v>14</v>
-      </c>
-      <c r="E11" s="45" t="s">
-        <v>52</v>
-      </c>
-      <c r="F11" s="45" t="s">
-        <v>94</v>
-      </c>
-      <c r="G11" s="46" t="s">
-        <v>124</v>
-      </c>
-      <c r="H11" s="45" t="s">
-        <v>153</v>
-      </c>
-      <c r="I11" s="45" t="s">
-        <v>225</v>
-      </c>
-      <c r="J11" s="45" t="s">
-        <v>244</v>
-      </c>
-      <c r="K11" s="58" t="s">
-        <v>182</v>
-      </c>
-      <c r="L11" s="59">
-        <v>1</v>
-      </c>
-      <c r="M11" s="59">
-        <f t="shared" ref="M11:M50" si="1">L11*5</f>
-        <v>5</v>
-      </c>
-      <c r="N11" s="45">
-        <v>20</v>
-      </c>
-      <c r="O11" s="62" t="s">
+      <c r="D11" s="71" t="s">
+        <v>285</v>
+      </c>
+      <c r="E11" s="67" t="s">
+        <v>60</v>
+      </c>
+      <c r="F11" s="61" t="s">
+        <v>97</v>
+      </c>
+      <c r="G11" s="67" t="s">
+        <v>131</v>
+      </c>
+      <c r="H11" s="61" t="s">
+        <v>152</v>
+      </c>
+      <c r="I11" s="61" t="s">
+        <v>225</v>
+      </c>
+      <c r="J11" s="61" t="s">
+        <v>173</v>
+      </c>
+      <c r="K11" s="68" t="s">
+        <v>183</v>
+      </c>
+      <c r="L11" s="61">
+        <v>51</v>
+      </c>
+      <c r="M11" s="61">
+        <f t="shared" ref="M11:M49" si="0">L11*5</f>
+        <v>255</v>
+      </c>
+      <c r="N11" s="61">
+        <v>300</v>
+      </c>
+      <c r="O11" s="69" t="s">
         <v>223</v>
       </c>
-      <c r="P11" s="47">
-        <v>1.7399999999999999E-2</v>
-      </c>
-      <c r="Q11" s="47">
-        <f t="shared" ref="Q11:Q50" si="2">P11*N11</f>
-        <v>0.34799999999999998</v>
-      </c>
-      <c r="R11" s="46"/>
-      <c r="S11" s="47"/>
-    </row>
-    <row r="12" spans="1:19" s="64" customFormat="1" ht="72.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P11" s="70">
+        <v>8.9999999999999993E-3</v>
+      </c>
+      <c r="Q11" s="70">
+        <f>P11*N11</f>
+        <v>2.6999999999999997</v>
+      </c>
+      <c r="R11" s="67"/>
+      <c r="S11" s="70"/>
+    </row>
+    <row r="12" spans="1:19" s="64" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="63"/>
       <c r="B12" s="37">
-        <f>ROW(B12) - ROW($B$9)</f>
+        <f t="shared" ref="B12:B48" si="1">ROW(B12) - ROW($B$9)</f>
         <v>3</v>
       </c>
       <c r="C12" s="53" t="s">
         <v>7</v>
       </c>
-      <c r="D12" s="71" t="s">
-        <v>260</v>
-      </c>
-      <c r="E12" s="67" t="s">
-        <v>60</v>
+      <c r="D12" s="110" t="s">
+        <v>15</v>
+      </c>
+      <c r="E12" s="61" t="s">
+        <v>53</v>
       </c>
       <c r="F12" s="61" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="G12" s="67" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="H12" s="61" t="s">
         <v>152</v>
@@ -2622,91 +2670,91 @@
         <v>225</v>
       </c>
       <c r="J12" s="61" t="s">
-        <v>173</v>
+        <v>245</v>
       </c>
       <c r="K12" s="68" t="s">
-        <v>183</v>
-      </c>
-      <c r="L12" s="61">
-        <v>43</v>
-      </c>
-      <c r="M12" s="61">
-        <f t="shared" si="1"/>
-        <v>215</v>
+        <v>184</v>
+      </c>
+      <c r="L12" s="111">
+        <v>12</v>
+      </c>
+      <c r="M12" s="111">
+        <f t="shared" si="0"/>
+        <v>60</v>
       </c>
       <c r="N12" s="61">
-        <v>250</v>
+        <v>100</v>
       </c>
       <c r="O12" s="69" t="s">
         <v>223</v>
       </c>
       <c r="P12" s="70">
-        <v>8.9999999999999993E-3</v>
+        <v>2.8E-3</v>
       </c>
       <c r="Q12" s="70">
-        <f>P12*N12</f>
-        <v>2.25</v>
+        <f t="shared" ref="Q12:Q49" si="2">P12*N12</f>
+        <v>0.27999999999999997</v>
       </c>
       <c r="R12" s="67"/>
       <c r="S12" s="70"/>
     </row>
-    <row r="13" spans="1:19" s="64" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:19" s="64" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="63"/>
       <c r="B13" s="37">
+        <f>ROW(B13) - ROW($B$9)</f>
+        <v>4</v>
+      </c>
+      <c r="C13" s="53" t="s">
+        <v>7</v>
+      </c>
+      <c r="D13" s="71" t="s">
+        <v>16</v>
+      </c>
+      <c r="E13" s="67" t="s">
+        <v>54</v>
+      </c>
+      <c r="F13" s="61" t="s">
+        <v>96</v>
+      </c>
+      <c r="G13" s="67" t="s">
+        <v>126</v>
+      </c>
+      <c r="H13" s="61" t="s">
+        <v>154</v>
+      </c>
+      <c r="I13" s="61" t="s">
+        <v>225</v>
+      </c>
+      <c r="J13" s="61" t="s">
+        <v>171</v>
+      </c>
+      <c r="K13" s="68" t="s">
+        <v>185</v>
+      </c>
+      <c r="L13" s="61">
+        <v>2</v>
+      </c>
+      <c r="M13" s="61">
         <f t="shared" si="0"/>
-        <v>4</v>
-      </c>
-      <c r="C13" s="52" t="s">
-        <v>7</v>
-      </c>
-      <c r="D13" s="72" t="s">
-        <v>15</v>
-      </c>
-      <c r="E13" s="45" t="s">
-        <v>53</v>
-      </c>
-      <c r="F13" s="45" t="s">
-        <v>95</v>
-      </c>
-      <c r="G13" s="46" t="s">
-        <v>125</v>
-      </c>
-      <c r="H13" s="45" t="s">
-        <v>152</v>
-      </c>
-      <c r="I13" s="45" t="s">
-        <v>225</v>
-      </c>
-      <c r="J13" s="45" t="s">
-        <v>245</v>
-      </c>
-      <c r="K13" s="58" t="s">
-        <v>184</v>
-      </c>
-      <c r="L13" s="59">
-        <v>12</v>
-      </c>
-      <c r="M13" s="59">
-        <f t="shared" si="1"/>
-        <v>60</v>
-      </c>
-      <c r="N13" s="45">
-        <v>100</v>
-      </c>
-      <c r="O13" s="62" t="s">
+        <v>10</v>
+      </c>
+      <c r="N13" s="61">
+        <v>11</v>
+      </c>
+      <c r="O13" s="69" t="s">
         <v>223</v>
       </c>
-      <c r="P13" s="47">
-        <v>2.8E-3</v>
-      </c>
-      <c r="Q13" s="47">
+      <c r="P13" s="70">
+        <v>1.2005999999999999</v>
+      </c>
+      <c r="Q13" s="70">
         <f t="shared" si="2"/>
-        <v>0.27999999999999997</v>
-      </c>
-      <c r="R13" s="46"/>
-      <c r="S13" s="47"/>
-    </row>
-    <row r="14" spans="1:19" s="64" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>13.206599999999998</v>
+      </c>
+      <c r="R13" s="67"/>
+      <c r="S13" s="70"/>
+    </row>
+    <row r="14" spans="1:19" s="64" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="63"/>
       <c r="B14" s="37">
         <f>ROW(B14) - ROW($B$9)</f>
@@ -2715,220 +2763,220 @@
       <c r="C14" s="53" t="s">
         <v>7</v>
       </c>
-      <c r="D14" s="71" t="s">
+      <c r="D14" s="110" t="s">
+        <v>261</v>
+      </c>
+      <c r="E14" s="61" t="s">
+        <v>55</v>
+      </c>
+      <c r="F14" s="61" t="s">
+        <v>93</v>
+      </c>
+      <c r="G14" s="74" t="s">
+        <v>127</v>
+      </c>
+      <c r="H14" s="61" t="s">
+        <v>152</v>
+      </c>
+      <c r="I14" s="61" t="s">
+        <v>262</v>
+      </c>
+      <c r="J14" s="61" t="s">
+        <v>263</v>
+      </c>
+      <c r="K14" s="68" t="s">
+        <v>186</v>
+      </c>
+      <c r="L14" s="111">
         <v>16</v>
       </c>
-      <c r="E14" s="67" t="s">
-        <v>54</v>
-      </c>
-      <c r="F14" s="61" t="s">
-        <v>96</v>
-      </c>
-      <c r="G14" s="67" t="s">
-        <v>126</v>
-      </c>
-      <c r="H14" s="61" t="s">
-        <v>154</v>
-      </c>
-      <c r="I14" s="61" t="s">
-        <v>225</v>
-      </c>
-      <c r="J14" s="61" t="s">
-        <v>171</v>
-      </c>
-      <c r="K14" s="68" t="s">
-        <v>185</v>
-      </c>
-      <c r="L14" s="61">
-        <v>2</v>
-      </c>
-      <c r="M14" s="61">
-        <f t="shared" si="1"/>
-        <v>10</v>
+      <c r="M14" s="111">
+        <f t="shared" si="0"/>
+        <v>80</v>
       </c>
       <c r="N14" s="61">
-        <v>11</v>
+        <v>100</v>
       </c>
       <c r="O14" s="69" t="s">
         <v>223</v>
       </c>
       <c r="P14" s="70">
-        <v>1.2005999999999999</v>
+        <v>2.5000000000000001E-3</v>
       </c>
       <c r="Q14" s="70">
         <f t="shared" si="2"/>
-        <v>13.206599999999998</v>
+        <v>0.25</v>
       </c>
       <c r="R14" s="67"/>
       <c r="S14" s="70"/>
     </row>
-    <row r="15" spans="1:19" s="64" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:19" s="64" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="63"/>
       <c r="B15" s="37">
-        <f>ROW(B15) - ROW($B$9)</f>
+        <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="C15" s="52" t="s">
+      <c r="C15" s="53" t="s">
         <v>7</v>
       </c>
-      <c r="D15" s="72" t="s">
-        <v>261</v>
-      </c>
-      <c r="E15" s="45" t="s">
-        <v>55</v>
-      </c>
-      <c r="F15" s="45" t="s">
-        <v>93</v>
-      </c>
-      <c r="G15" s="73" t="s">
-        <v>127</v>
-      </c>
-      <c r="H15" s="45" t="s">
-        <v>152</v>
-      </c>
-      <c r="I15" s="45" t="s">
-        <v>262</v>
-      </c>
-      <c r="J15" s="45" t="s">
-        <v>263</v>
-      </c>
-      <c r="K15" s="58" t="s">
-        <v>186</v>
-      </c>
-      <c r="L15" s="59">
-        <v>16</v>
-      </c>
-      <c r="M15" s="59">
-        <f t="shared" si="1"/>
-        <v>80</v>
-      </c>
-      <c r="N15" s="45">
-        <v>100</v>
-      </c>
-      <c r="O15" s="62" t="s">
+      <c r="D15" s="71" t="s">
+        <v>17</v>
+      </c>
+      <c r="E15" s="67" t="s">
+        <v>56</v>
+      </c>
+      <c r="F15" s="61" t="s">
+        <v>94</v>
+      </c>
+      <c r="G15" s="67" t="s">
+        <v>128</v>
+      </c>
+      <c r="H15" s="61" t="s">
+        <v>155</v>
+      </c>
+      <c r="I15" s="61" t="s">
+        <v>225</v>
+      </c>
+      <c r="J15" s="61" t="s">
+        <v>246</v>
+      </c>
+      <c r="K15" s="68" t="s">
+        <v>187</v>
+      </c>
+      <c r="L15" s="61">
+        <v>1</v>
+      </c>
+      <c r="M15" s="61">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="N15" s="61">
+        <v>10</v>
+      </c>
+      <c r="O15" s="69" t="s">
         <v>223</v>
       </c>
-      <c r="P15" s="47">
-        <v>2.5000000000000001E-3</v>
-      </c>
-      <c r="Q15" s="47">
+      <c r="P15" s="70">
+        <v>3.7699999999999997E-2</v>
+      </c>
+      <c r="Q15" s="70">
         <f t="shared" si="2"/>
-        <v>0.25</v>
-      </c>
-      <c r="R15" s="46"/>
-      <c r="S15" s="47"/>
-    </row>
-    <row r="16" spans="1:19" s="64" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>0.377</v>
+      </c>
+      <c r="R15" s="67"/>
+      <c r="S15" s="70"/>
+    </row>
+    <row r="16" spans="1:19" s="64" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="63"/>
       <c r="B16" s="37">
-        <f t="shared" si="0"/>
+        <f>ROW(B16) - ROW($B$9)</f>
         <v>7</v>
       </c>
       <c r="C16" s="53" t="s">
         <v>7</v>
       </c>
-      <c r="D16" s="71" t="s">
-        <v>17</v>
-      </c>
-      <c r="E16" s="67" t="s">
-        <v>56</v>
+      <c r="D16" s="110" t="s">
+        <v>18</v>
+      </c>
+      <c r="E16" s="61" t="s">
+        <v>57</v>
       </c>
       <c r="F16" s="61" t="s">
         <v>94</v>
       </c>
       <c r="G16" s="67" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H16" s="61" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="I16" s="61" t="s">
         <v>225</v>
       </c>
       <c r="J16" s="61" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="K16" s="68" t="s">
-        <v>187</v>
-      </c>
-      <c r="L16" s="61">
-        <v>1</v>
-      </c>
-      <c r="M16" s="61">
-        <f t="shared" si="1"/>
-        <v>5</v>
+        <v>188</v>
+      </c>
+      <c r="L16" s="111">
+        <v>6</v>
+      </c>
+      <c r="M16" s="111">
+        <f t="shared" si="0"/>
+        <v>30</v>
       </c>
       <c r="N16" s="61">
-        <v>10</v>
+        <v>100</v>
       </c>
       <c r="O16" s="69" t="s">
         <v>223</v>
       </c>
       <c r="P16" s="70">
-        <v>3.7699999999999997E-2</v>
+        <v>2.7000000000000001E-3</v>
       </c>
       <c r="Q16" s="70">
         <f t="shared" si="2"/>
-        <v>0.377</v>
+        <v>0.27</v>
       </c>
       <c r="R16" s="67"/>
       <c r="S16" s="70"/>
     </row>
-    <row r="17" spans="1:19" s="64" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:19" s="64" customFormat="1" ht="96.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="63"/>
       <c r="B17" s="37">
         <f>ROW(B17) - ROW($B$9)</f>
         <v>8</v>
       </c>
-      <c r="C17" s="52" t="s">
+      <c r="C17" s="53" t="s">
         <v>7</v>
       </c>
-      <c r="D17" s="72" t="s">
-        <v>18</v>
-      </c>
-      <c r="E17" s="45" t="s">
-        <v>57</v>
-      </c>
-      <c r="F17" s="45" t="s">
-        <v>94</v>
-      </c>
-      <c r="G17" s="46" t="s">
-        <v>129</v>
-      </c>
-      <c r="H17" s="45" t="s">
+      <c r="D17" s="71" t="s">
+        <v>286</v>
+      </c>
+      <c r="E17" s="67" t="s">
+        <v>63</v>
+      </c>
+      <c r="F17" s="61" t="s">
+        <v>97</v>
+      </c>
+      <c r="G17" s="67" t="s">
+        <v>135</v>
+      </c>
+      <c r="H17" s="61" t="s">
         <v>152</v>
       </c>
-      <c r="I17" s="45" t="s">
-        <v>225</v>
-      </c>
-      <c r="J17" s="45" t="s">
-        <v>247</v>
-      </c>
-      <c r="K17" s="58" t="s">
-        <v>188</v>
-      </c>
-      <c r="L17" s="59">
-        <v>6</v>
-      </c>
-      <c r="M17" s="59">
-        <f t="shared" si="1"/>
-        <v>30</v>
-      </c>
-      <c r="N17" s="45">
-        <v>100</v>
-      </c>
-      <c r="O17" s="62" t="s">
+      <c r="I17" s="61" t="s">
+        <v>225</v>
+      </c>
+      <c r="J17" s="61" t="s">
+        <v>175</v>
+      </c>
+      <c r="K17" s="68" t="s">
+        <v>186</v>
+      </c>
+      <c r="L17" s="61">
+        <v>48</v>
+      </c>
+      <c r="M17" s="61">
+        <f>L17*5</f>
+        <v>240</v>
+      </c>
+      <c r="N17" s="61">
+        <v>300</v>
+      </c>
+      <c r="O17" s="69" t="s">
         <v>223</v>
       </c>
-      <c r="P17" s="47">
-        <v>2.7000000000000001E-3</v>
-      </c>
-      <c r="Q17" s="47">
-        <f t="shared" si="2"/>
-        <v>0.27</v>
-      </c>
-      <c r="R17" s="46"/>
-      <c r="S17" s="47"/>
+      <c r="P17" s="70">
+        <v>1.1000000000000001E-3</v>
+      </c>
+      <c r="Q17" s="70">
+        <f>P17*N17</f>
+        <v>0.33</v>
+      </c>
+      <c r="R17" s="67"/>
+      <c r="S17" s="70"/>
     </row>
     <row r="18" spans="1:19" s="64" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="63"/>
@@ -2939,7 +2987,7 @@
       <c r="C18" s="53" t="s">
         <v>7</v>
       </c>
-      <c r="D18" s="71" t="s">
+      <c r="D18" s="110" t="s">
         <v>277</v>
       </c>
       <c r="E18" s="67" t="s">
@@ -2948,17 +2996,17 @@
       <c r="F18" s="61" t="s">
         <v>93</v>
       </c>
-      <c r="G18" s="74" t="s">
-        <v>134</v>
+      <c r="G18" s="61" t="s">
+        <v>264</v>
       </c>
       <c r="H18" s="61" t="s">
         <v>156</v>
       </c>
       <c r="I18" s="61" t="s">
-        <v>264</v>
+        <v>225</v>
       </c>
       <c r="J18" s="61" t="s">
-        <v>265</v>
+        <v>287</v>
       </c>
       <c r="K18" s="68" t="s">
         <v>189</v>
@@ -2967,7 +3015,7 @@
         <v>11</v>
       </c>
       <c r="M18" s="61">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>55</v>
       </c>
       <c r="N18" s="61">
@@ -2992,60 +3040,60 @@
         <f>ROW(B19) - ROW($B$9)</f>
         <v>10</v>
       </c>
-      <c r="C19" s="52" t="s">
+      <c r="C19" s="53" t="s">
         <v>7</v>
       </c>
-      <c r="D19" s="72" t="s">
+      <c r="D19" s="110" t="s">
         <v>19</v>
       </c>
-      <c r="E19" s="45" t="s">
+      <c r="E19" s="61" t="s">
         <v>59</v>
       </c>
-      <c r="F19" s="45" t="s">
+      <c r="F19" s="61" t="s">
         <v>93</v>
       </c>
-      <c r="G19" s="46" t="s">
+      <c r="G19" s="67" t="s">
         <v>130</v>
       </c>
-      <c r="H19" s="45" t="s">
+      <c r="H19" s="61" t="s">
         <v>152</v>
       </c>
-      <c r="I19" s="45" t="s">
-        <v>225</v>
-      </c>
-      <c r="J19" s="45" t="s">
+      <c r="I19" s="61" t="s">
+        <v>225</v>
+      </c>
+      <c r="J19" s="61" t="s">
         <v>172</v>
       </c>
-      <c r="K19" s="58" t="s">
+      <c r="K19" s="68" t="s">
         <v>190</v>
       </c>
-      <c r="L19" s="59">
+      <c r="L19" s="111">
         <v>4</v>
       </c>
-      <c r="M19" s="59">
-        <f t="shared" si="1"/>
+      <c r="M19" s="111">
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="N19" s="45">
+      <c r="N19" s="61">
         <v>100</v>
       </c>
-      <c r="O19" s="62" t="s">
+      <c r="O19" s="69" t="s">
         <v>223</v>
       </c>
-      <c r="P19" s="47">
+      <c r="P19" s="70">
         <v>2.5000000000000001E-3</v>
       </c>
-      <c r="Q19" s="47">
+      <c r="Q19" s="70">
         <f t="shared" si="2"/>
         <v>0.25</v>
       </c>
-      <c r="R19" s="46"/>
-      <c r="S19" s="47"/>
+      <c r="R19" s="67"/>
+      <c r="S19" s="70"/>
     </row>
     <row r="20" spans="1:19" s="64" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="63"/>
       <c r="B20" s="37">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>11</v>
       </c>
       <c r="C20" s="53" t="s">
@@ -3079,7 +3127,7 @@
         <v>1</v>
       </c>
       <c r="M20" s="61">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="N20" s="61">
@@ -3104,108 +3152,108 @@
         <f>ROW(B21) - ROW($B$9)</f>
         <v>12</v>
       </c>
-      <c r="C21" s="52" t="s">
+      <c r="C21" s="53" t="s">
         <v>7</v>
       </c>
-      <c r="D21" s="72" t="s">
+      <c r="D21" s="110" t="s">
         <v>21</v>
       </c>
-      <c r="E21" s="45" t="s">
+      <c r="E21" s="61" t="s">
         <v>62</v>
       </c>
-      <c r="F21" s="45" t="s">
+      <c r="F21" s="61" t="s">
         <v>93</v>
       </c>
-      <c r="G21" s="46" t="s">
+      <c r="G21" s="67" t="s">
         <v>133</v>
       </c>
-      <c r="H21" s="45" t="s">
+      <c r="H21" s="61" t="s">
         <v>152</v>
       </c>
-      <c r="I21" s="45" t="s">
-        <v>225</v>
-      </c>
-      <c r="J21" s="45" t="s">
+      <c r="I21" s="61" t="s">
+        <v>225</v>
+      </c>
+      <c r="J21" s="61" t="s">
         <v>174</v>
       </c>
-      <c r="K21" s="58" t="s">
+      <c r="K21" s="68" t="s">
         <v>192</v>
       </c>
-      <c r="L21" s="59">
+      <c r="L21" s="111">
         <v>8</v>
       </c>
-      <c r="M21" s="59">
-        <f t="shared" si="1"/>
+      <c r="M21" s="111">
+        <f t="shared" si="0"/>
         <v>40</v>
       </c>
-      <c r="N21" s="45">
+      <c r="N21" s="61">
         <v>100</v>
       </c>
-      <c r="O21" s="62" t="s">
+      <c r="O21" s="69" t="s">
         <v>223</v>
       </c>
-      <c r="P21" s="47">
+      <c r="P21" s="70">
         <v>2.7000000000000001E-3</v>
       </c>
-      <c r="Q21" s="47">
+      <c r="Q21" s="70">
         <f t="shared" si="2"/>
         <v>0.27</v>
       </c>
-      <c r="R21" s="46"/>
-      <c r="S21" s="47"/>
-    </row>
-    <row r="22" spans="1:19" s="64" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R21" s="67"/>
+      <c r="S21" s="70"/>
+    </row>
+    <row r="22" spans="1:19" s="64" customFormat="1" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="63"/>
       <c r="B22" s="37">
-        <f>ROW(B22) - ROW($B$9)</f>
+        <f t="shared" si="1"/>
         <v>13</v>
       </c>
       <c r="C22" s="53" t="s">
-        <v>7</v>
-      </c>
-      <c r="D22" s="71" t="s">
-        <v>22</v>
-      </c>
-      <c r="E22" s="67" t="s">
-        <v>63</v>
+        <v>201</v>
+      </c>
+      <c r="D22" s="110" t="s">
+        <v>24</v>
+      </c>
+      <c r="E22" s="61" t="s">
+        <v>65</v>
       </c>
       <c r="F22" s="61" t="s">
-        <v>97</v>
+        <v>224</v>
       </c>
       <c r="G22" s="67" t="s">
-        <v>135</v>
+        <v>99</v>
       </c>
       <c r="H22" s="61" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="I22" s="61" t="s">
         <v>225</v>
       </c>
       <c r="J22" s="61" t="s">
-        <v>175</v>
+        <v>226</v>
       </c>
       <c r="K22" s="68" t="s">
-        <v>186</v>
-      </c>
-      <c r="L22" s="61">
-        <v>8</v>
-      </c>
-      <c r="M22" s="61">
-        <f t="shared" si="1"/>
-        <v>40</v>
+        <v>225</v>
+      </c>
+      <c r="L22" s="111">
+        <v>1</v>
+      </c>
+      <c r="M22" s="111">
+        <f t="shared" si="0"/>
+        <v>5</v>
       </c>
       <c r="N22" s="61">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="O22" s="69" t="s">
         <v>223</v>
       </c>
       <c r="P22" s="70">
-        <v>1.1000000000000001E-3</v>
+        <v>3.9800000000000002E-2</v>
       </c>
       <c r="Q22" s="70">
         <f t="shared" si="2"/>
-        <v>0.11</v>
+        <v>0.39800000000000002</v>
       </c>
       <c r="R22" s="67"/>
       <c r="S22" s="70"/>
@@ -3213,582 +3261,581 @@
     <row r="23" spans="1:19" s="64" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="63"/>
       <c r="B23" s="37">
+        <f>ROW(B23) - ROW($B$9)</f>
+        <v>14</v>
+      </c>
+      <c r="C23" s="53" t="s">
+        <v>201</v>
+      </c>
+      <c r="D23" s="71" t="s">
+        <v>25</v>
+      </c>
+      <c r="E23" s="67" t="s">
+        <v>66</v>
+      </c>
+      <c r="F23" s="61" t="s">
+        <v>100</v>
+      </c>
+      <c r="G23" s="67" t="s">
+        <v>137</v>
+      </c>
+      <c r="H23" s="61" t="s">
+        <v>158</v>
+      </c>
+      <c r="I23" s="61" t="s">
+        <v>225</v>
+      </c>
+      <c r="J23" s="61" t="s">
+        <v>227</v>
+      </c>
+      <c r="K23" s="68" t="s">
+        <v>225</v>
+      </c>
+      <c r="L23" s="61">
+        <v>1</v>
+      </c>
+      <c r="M23" s="61">
         <f t="shared" si="0"/>
-        <v>14</v>
-      </c>
-      <c r="C23" s="52" t="s">
-        <v>7</v>
-      </c>
-      <c r="D23" s="72" t="s">
-        <v>23</v>
-      </c>
-      <c r="E23" s="45" t="s">
-        <v>64</v>
-      </c>
-      <c r="F23" s="45" t="s">
-        <v>98</v>
-      </c>
-      <c r="G23" s="46" t="s">
-        <v>136</v>
-      </c>
-      <c r="H23" s="45" t="s">
-        <v>155</v>
-      </c>
-      <c r="I23" s="45" t="s">
-        <v>225</v>
-      </c>
-      <c r="J23" s="45" t="s">
-        <v>249</v>
-      </c>
-      <c r="K23" s="58" t="s">
-        <v>189</v>
-      </c>
-      <c r="L23" s="59">
-        <v>8</v>
-      </c>
-      <c r="M23" s="59">
-        <f t="shared" si="1"/>
-        <v>40</v>
-      </c>
-      <c r="N23" s="45">
-        <v>45</v>
-      </c>
-      <c r="O23" s="62" t="s">
+        <v>5</v>
+      </c>
+      <c r="N23" s="61">
+        <v>10</v>
+      </c>
+      <c r="O23" s="69" t="s">
         <v>223</v>
       </c>
-      <c r="P23" s="47">
-        <v>8.9399999999999993E-2</v>
-      </c>
-      <c r="Q23" s="47">
+      <c r="P23" s="70">
+        <v>3.1800000000000002E-2</v>
+      </c>
+      <c r="Q23" s="70">
         <f t="shared" si="2"/>
-        <v>4.0229999999999997</v>
-      </c>
-      <c r="R23" s="46"/>
-      <c r="S23" s="47"/>
-    </row>
-    <row r="24" spans="1:19" s="64" customFormat="1" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>0.318</v>
+      </c>
+      <c r="R23" s="67"/>
+      <c r="S23" s="70"/>
+    </row>
+    <row r="24" spans="1:19" s="64" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="63"/>
       <c r="B24" s="37">
-        <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="C24" s="52" t="s">
-        <v>201</v>
-      </c>
-      <c r="D24" s="72" t="s">
-        <v>24</v>
-      </c>
-      <c r="E24" s="45" t="s">
-        <v>65</v>
-      </c>
-      <c r="F24" s="45" t="s">
-        <v>224</v>
-      </c>
-      <c r="G24" s="46" t="s">
-        <v>99</v>
-      </c>
-      <c r="H24" s="45" t="s">
-        <v>157</v>
-      </c>
-      <c r="I24" s="45" t="s">
-        <v>225</v>
-      </c>
-      <c r="J24" s="45" t="s">
-        <v>226</v>
-      </c>
-      <c r="K24" s="58" t="s">
-        <v>225</v>
-      </c>
-      <c r="L24" s="59">
-        <v>1</v>
-      </c>
-      <c r="M24" s="59">
-        <f t="shared" si="1"/>
-        <v>5</v>
-      </c>
-      <c r="N24" s="45">
+      <c r="C24" s="53" t="s">
+        <v>288</v>
+      </c>
+      <c r="D24" s="109" t="s">
+        <v>289</v>
+      </c>
+      <c r="E24" s="109" t="s">
+        <v>290</v>
+      </c>
+      <c r="F24" s="109" t="s">
+        <v>291</v>
+      </c>
+      <c r="G24" s="109" t="s">
+        <v>292</v>
+      </c>
+      <c r="H24" s="109" t="s">
+        <v>293</v>
+      </c>
+      <c r="I24" s="109" t="s">
+        <v>225</v>
+      </c>
+      <c r="J24" s="109" t="s">
+        <v>294</v>
+      </c>
+      <c r="K24" s="109" t="s">
+        <v>225</v>
+      </c>
+      <c r="L24" s="109">
+        <v>2</v>
+      </c>
+      <c r="M24" s="111">
+        <f>L24*5</f>
         <v>10</v>
       </c>
-      <c r="O24" s="62" t="s">
+      <c r="N24" s="61">
+        <v>20</v>
+      </c>
+      <c r="O24" s="69" t="s">
         <v>223</v>
       </c>
-      <c r="P24" s="47">
-        <v>3.9800000000000002E-2</v>
-      </c>
-      <c r="Q24" s="47">
-        <f t="shared" si="2"/>
-        <v>0.39800000000000002</v>
-      </c>
-      <c r="R24" s="46"/>
-      <c r="S24" s="47"/>
-    </row>
-    <row r="25" spans="1:19" s="64" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P24" s="70">
+        <v>3.2199999999999999E-2</v>
+      </c>
+      <c r="Q24" s="70">
+        <f>P24*N24</f>
+        <v>0.64400000000000002</v>
+      </c>
+      <c r="R24" s="67"/>
+      <c r="S24" s="70"/>
+    </row>
+    <row r="25" spans="1:19" s="64" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="63"/>
       <c r="B25" s="37">
-        <f>ROW(B25) - ROW($B$9)</f>
+        <f t="shared" si="1"/>
         <v>16</v>
       </c>
       <c r="C25" s="53" t="s">
-        <v>201</v>
-      </c>
-      <c r="D25" s="71" t="s">
-        <v>25</v>
-      </c>
-      <c r="E25" s="67" t="s">
-        <v>66</v>
+        <v>202</v>
+      </c>
+      <c r="D25" s="110" t="s">
+        <v>26</v>
+      </c>
+      <c r="E25" s="61" t="s">
+        <v>67</v>
       </c>
       <c r="F25" s="61" t="s">
-        <v>100</v>
-      </c>
-      <c r="G25" s="67" t="s">
-        <v>137</v>
+        <v>101</v>
+      </c>
+      <c r="G25" s="74" t="s">
+        <v>138</v>
       </c>
       <c r="H25" s="61" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I25" s="61" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="J25" s="61" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="K25" s="68" t="s">
         <v>225</v>
       </c>
-      <c r="L25" s="61">
+      <c r="L25" s="111">
         <v>1</v>
       </c>
-      <c r="M25" s="61">
-        <f t="shared" si="1"/>
+      <c r="M25" s="111">
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="N25" s="61">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="O25" s="69" t="s">
         <v>223</v>
       </c>
       <c r="P25" s="70">
-        <v>3.1800000000000002E-2</v>
+        <v>2.8000000000000001E-2</v>
       </c>
       <c r="Q25" s="70">
         <f t="shared" si="2"/>
-        <v>0.318</v>
+        <v>0.56000000000000005</v>
       </c>
       <c r="R25" s="67"/>
       <c r="S25" s="70"/>
     </row>
-    <row r="26" spans="1:19" s="64" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:19" s="64" customFormat="1" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="63"/>
       <c r="B26" s="37">
+        <f>ROW(B26) - ROW($B$9)</f>
+        <v>17</v>
+      </c>
+      <c r="C26" s="53" t="s">
+        <v>8</v>
+      </c>
+      <c r="D26" s="71" t="s">
+        <v>27</v>
+      </c>
+      <c r="E26" s="67" t="s">
+        <v>68</v>
+      </c>
+      <c r="F26" s="61" t="s">
+        <v>230</v>
+      </c>
+      <c r="G26" s="67" t="s">
+        <v>102</v>
+      </c>
+      <c r="H26" s="61" t="s">
+        <v>160</v>
+      </c>
+      <c r="I26" s="61" t="s">
+        <v>225</v>
+      </c>
+      <c r="J26" s="61" t="s">
+        <v>176</v>
+      </c>
+      <c r="K26" s="68" t="s">
+        <v>225</v>
+      </c>
+      <c r="L26" s="61">
+        <v>1</v>
+      </c>
+      <c r="M26" s="61">
         <f t="shared" si="0"/>
-        <v>17</v>
-      </c>
-      <c r="C26" s="52" t="s">
-        <v>202</v>
-      </c>
-      <c r="D26" s="72" t="s">
-        <v>26</v>
-      </c>
-      <c r="E26" s="45" t="s">
-        <v>67</v>
-      </c>
-      <c r="F26" s="45" t="s">
-        <v>101</v>
-      </c>
-      <c r="G26" s="73" t="s">
-        <v>138</v>
-      </c>
-      <c r="H26" s="45" t="s">
-        <v>159</v>
-      </c>
-      <c r="I26" s="45" t="s">
-        <v>228</v>
-      </c>
-      <c r="J26" s="45" t="s">
-        <v>229</v>
-      </c>
-      <c r="K26" s="58" t="s">
-        <v>225</v>
-      </c>
-      <c r="L26" s="59">
-        <v>1</v>
-      </c>
-      <c r="M26" s="59">
-        <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="N26" s="45">
-        <v>20</v>
-      </c>
-      <c r="O26" s="62" t="s">
+      <c r="N26" s="61">
+        <v>10</v>
+      </c>
+      <c r="O26" s="69" t="s">
         <v>223</v>
       </c>
-      <c r="P26" s="47">
-        <v>2.8000000000000001E-2</v>
-      </c>
-      <c r="Q26" s="47">
+      <c r="P26" s="70">
+        <v>5.5599999999999997E-2</v>
+      </c>
+      <c r="Q26" s="70">
         <f t="shared" si="2"/>
-        <v>0.56000000000000005</v>
-      </c>
-      <c r="R26" s="46"/>
-      <c r="S26" s="47"/>
-    </row>
-    <row r="27" spans="1:19" s="64" customFormat="1" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>0.55599999999999994</v>
+      </c>
+      <c r="R26" s="67"/>
+      <c r="S26" s="70"/>
+    </row>
+    <row r="27" spans="1:19" s="64" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="63"/>
       <c r="B27" s="37">
-        <f>ROW(B27) - ROW($B$9)</f>
+        <f t="shared" si="1"/>
         <v>18</v>
       </c>
       <c r="C27" s="53" t="s">
-        <v>8</v>
-      </c>
-      <c r="D27" s="71" t="s">
-        <v>27</v>
-      </c>
-      <c r="E27" s="67" t="s">
-        <v>68</v>
+        <v>9</v>
+      </c>
+      <c r="D27" s="110" t="s">
+        <v>28</v>
+      </c>
+      <c r="E27" s="61" t="s">
+        <v>69</v>
       </c>
       <c r="F27" s="61" t="s">
         <v>230</v>
       </c>
       <c r="G27" s="67" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="H27" s="61" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="I27" s="61" t="s">
         <v>225</v>
       </c>
       <c r="J27" s="61" t="s">
-        <v>176</v>
+        <v>225</v>
       </c>
       <c r="K27" s="68" t="s">
         <v>225</v>
       </c>
-      <c r="L27" s="61">
-        <v>1</v>
-      </c>
-      <c r="M27" s="61">
-        <f t="shared" si="1"/>
-        <v>5</v>
+      <c r="L27" s="111">
+        <v>8</v>
+      </c>
+      <c r="M27" s="111">
+        <f t="shared" si="0"/>
+        <v>40</v>
       </c>
       <c r="N27" s="61">
-        <v>10</v>
+        <v>45</v>
       </c>
       <c r="O27" s="69" t="s">
-        <v>223</v>
+        <v>276</v>
       </c>
       <c r="P27" s="70">
-        <v>5.5599999999999997E-2</v>
+        <v>0.84699999999999998</v>
       </c>
       <c r="Q27" s="70">
         <f t="shared" si="2"/>
-        <v>0.55599999999999994</v>
-      </c>
-      <c r="R27" s="67"/>
+        <v>38.115000000000002</v>
+      </c>
+      <c r="R27" s="95"/>
       <c r="S27" s="70"/>
     </row>
     <row r="28" spans="1:19" s="64" customFormat="1" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="63"/>
       <c r="B28" s="37">
+        <f>ROW(B28) - ROW($B$9)</f>
+        <v>19</v>
+      </c>
+      <c r="C28" s="53" t="s">
+        <v>9</v>
+      </c>
+      <c r="D28" s="71" t="s">
+        <v>29</v>
+      </c>
+      <c r="E28" s="67" t="s">
+        <v>70</v>
+      </c>
+      <c r="F28" s="61" t="s">
+        <v>230</v>
+      </c>
+      <c r="G28" s="67" t="s">
+        <v>104</v>
+      </c>
+      <c r="H28" s="61" t="s">
+        <v>161</v>
+      </c>
+      <c r="I28" s="61" t="s">
+        <v>225</v>
+      </c>
+      <c r="J28" s="61" t="s">
+        <v>225</v>
+      </c>
+      <c r="K28" s="68" t="s">
+        <v>225</v>
+      </c>
+      <c r="L28" s="61">
+        <v>4</v>
+      </c>
+      <c r="M28" s="61">
         <f t="shared" si="0"/>
-        <v>19</v>
-      </c>
-      <c r="C28" s="52" t="s">
-        <v>9</v>
-      </c>
-      <c r="D28" s="72" t="s">
-        <v>28</v>
-      </c>
-      <c r="E28" s="45" t="s">
-        <v>69</v>
-      </c>
-      <c r="F28" s="45" t="s">
-        <v>230</v>
-      </c>
-      <c r="G28" s="46" t="s">
-        <v>103</v>
-      </c>
-      <c r="H28" s="45" t="s">
-        <v>161</v>
-      </c>
-      <c r="I28" s="45" t="s">
-        <v>225</v>
-      </c>
-      <c r="J28" s="45" t="s">
-        <v>225</v>
-      </c>
-      <c r="K28" s="58" t="s">
-        <v>225</v>
-      </c>
-      <c r="L28" s="59">
-        <v>8</v>
-      </c>
-      <c r="M28" s="59">
-        <f t="shared" si="1"/>
-        <v>40</v>
-      </c>
-      <c r="N28" s="45">
-        <v>45</v>
-      </c>
-      <c r="O28" s="62" t="s">
-        <v>276</v>
-      </c>
-      <c r="P28" s="47">
-        <v>0.84699999999999998</v>
-      </c>
-      <c r="Q28" s="47">
+        <v>20</v>
+      </c>
+      <c r="N28" s="61">
+        <v>25</v>
+      </c>
+      <c r="O28" s="69" t="s">
+        <v>231</v>
+      </c>
+      <c r="P28" s="70">
+        <v>2</v>
+      </c>
+      <c r="Q28" s="70">
         <f t="shared" si="2"/>
-        <v>38.115000000000002</v>
-      </c>
-      <c r="R28" s="89"/>
-      <c r="S28" s="47"/>
-    </row>
-    <row r="29" spans="1:19" s="64" customFormat="1" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>50</v>
+      </c>
+      <c r="R28" s="95" t="s">
+        <v>269</v>
+      </c>
+      <c r="S28" s="70"/>
+    </row>
+    <row r="29" spans="1:19" s="64" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="63"/>
       <c r="B29" s="37">
-        <f>ROW(B29) - ROW($B$9)</f>
-        <v>20</v>
-      </c>
-      <c r="C29" s="53" t="s">
-        <v>9</v>
-      </c>
-      <c r="D29" s="71" t="s">
-        <v>29</v>
-      </c>
-      <c r="E29" s="67" t="s">
-        <v>70</v>
-      </c>
-      <c r="F29" s="61" t="s">
-        <v>230</v>
-      </c>
-      <c r="G29" s="67" t="s">
-        <v>104</v>
-      </c>
-      <c r="H29" s="61" t="s">
-        <v>161</v>
-      </c>
-      <c r="I29" s="61" t="s">
-        <v>225</v>
-      </c>
-      <c r="J29" s="61" t="s">
-        <v>225</v>
-      </c>
-      <c r="K29" s="68" t="s">
-        <v>225</v>
-      </c>
-      <c r="L29" s="61">
-        <v>4</v>
-      </c>
-      <c r="M29" s="61">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
+      <c r="C29" s="53" t="s">
+        <v>202</v>
+      </c>
+      <c r="D29" s="110" t="s">
+        <v>30</v>
+      </c>
+      <c r="E29" s="61" t="s">
+        <v>71</v>
+      </c>
+      <c r="F29" s="61" t="s">
+        <v>105</v>
+      </c>
+      <c r="G29" s="74">
+        <v>61300611121</v>
+      </c>
+      <c r="H29" s="61" t="s">
+        <v>162</v>
+      </c>
+      <c r="I29" s="61" t="s">
+        <v>283</v>
+      </c>
+      <c r="J29" s="61" t="s">
+        <v>282</v>
+      </c>
+      <c r="K29" s="68" t="s">
+        <v>225</v>
+      </c>
+      <c r="L29" s="111">
+        <v>1</v>
+      </c>
+      <c r="M29" s="111">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
       <c r="N29" s="61">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="O29" s="69" t="s">
-        <v>231</v>
+        <v>223</v>
       </c>
       <c r="P29" s="70">
-        <v>2</v>
+        <v>3.3000000000000002E-2</v>
       </c>
       <c r="Q29" s="70">
         <f t="shared" si="2"/>
-        <v>50</v>
-      </c>
-      <c r="R29" s="95" t="s">
-        <v>269</v>
-      </c>
+        <v>0.66</v>
+      </c>
+      <c r="R29" s="67"/>
       <c r="S29" s="70"/>
     </row>
-    <row r="30" spans="1:19" s="64" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:19" s="64" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="63"/>
       <c r="B30" s="37">
+        <f>ROW(B30) - ROW($B$9)</f>
+        <v>21</v>
+      </c>
+      <c r="C30" s="53" t="s">
+        <v>203</v>
+      </c>
+      <c r="D30" s="90" t="s">
+        <v>31</v>
+      </c>
+      <c r="E30" s="74" t="s">
+        <v>72</v>
+      </c>
+      <c r="F30" s="91" t="s">
+        <v>230</v>
+      </c>
+      <c r="G30" s="74" t="s">
+        <v>106</v>
+      </c>
+      <c r="H30" s="91" t="s">
+        <v>225</v>
+      </c>
+      <c r="I30" s="91" t="s">
+        <v>225</v>
+      </c>
+      <c r="J30" s="91" t="s">
+        <v>225</v>
+      </c>
+      <c r="K30" s="92" t="s">
+        <v>225</v>
+      </c>
+      <c r="L30" s="91">
+        <v>5</v>
+      </c>
+      <c r="M30" s="91">
         <f t="shared" si="0"/>
-        <v>21</v>
-      </c>
-      <c r="C30" s="52" t="s">
-        <v>202</v>
-      </c>
-      <c r="D30" s="72" t="s">
-        <v>30</v>
-      </c>
-      <c r="E30" s="45" t="s">
-        <v>71</v>
-      </c>
-      <c r="F30" s="45" t="s">
-        <v>105</v>
-      </c>
-      <c r="G30" s="73">
-        <v>61300611121</v>
-      </c>
-      <c r="H30" s="45" t="s">
-        <v>162</v>
-      </c>
-      <c r="I30" s="45" t="s">
-        <v>283</v>
-      </c>
-      <c r="J30" s="45" t="s">
-        <v>282</v>
-      </c>
-      <c r="K30" s="58" t="s">
-        <v>225</v>
-      </c>
-      <c r="L30" s="59">
-        <v>1</v>
-      </c>
-      <c r="M30" s="59">
-        <f t="shared" si="1"/>
-        <v>5</v>
-      </c>
-      <c r="N30" s="45">
-        <v>20</v>
-      </c>
-      <c r="O30" s="62" t="s">
-        <v>223</v>
-      </c>
-      <c r="P30" s="47">
-        <v>3.3000000000000002E-2</v>
-      </c>
-      <c r="Q30" s="47">
-        <f t="shared" si="2"/>
-        <v>0.66</v>
-      </c>
-      <c r="R30" s="46"/>
-      <c r="S30" s="47"/>
+        <v>25</v>
+      </c>
+      <c r="N30" s="91"/>
+      <c r="O30" s="93" t="s">
+        <v>225</v>
+      </c>
+      <c r="P30" s="94" t="s">
+        <v>225</v>
+      </c>
+      <c r="Q30" s="94" t="s">
+        <v>225</v>
+      </c>
+      <c r="R30" s="74"/>
+      <c r="S30" s="94"/>
     </row>
     <row r="31" spans="1:19" s="64" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="63"/>
       <c r="B31" s="37">
-        <f>ROW(B31) - ROW($B$9)</f>
+        <f t="shared" si="1"/>
         <v>22</v>
       </c>
       <c r="C31" s="53" t="s">
-        <v>203</v>
-      </c>
-      <c r="D31" s="90" t="s">
-        <v>31</v>
-      </c>
-      <c r="E31" s="74" t="s">
-        <v>72</v>
-      </c>
-      <c r="F31" s="91" t="s">
-        <v>230</v>
+        <v>204</v>
+      </c>
+      <c r="D31" s="110" t="s">
+        <v>32</v>
+      </c>
+      <c r="E31" s="61" t="s">
+        <v>73</v>
+      </c>
+      <c r="F31" s="61" t="s">
+        <v>107</v>
       </c>
       <c r="G31" s="74" t="s">
-        <v>106</v>
-      </c>
-      <c r="H31" s="91" t="s">
-        <v>225</v>
-      </c>
-      <c r="I31" s="91" t="s">
-        <v>225</v>
-      </c>
-      <c r="J31" s="91" t="s">
-        <v>225</v>
-      </c>
-      <c r="K31" s="92" t="s">
-        <v>225</v>
-      </c>
-      <c r="L31" s="91">
-        <v>5</v>
-      </c>
-      <c r="M31" s="91">
-        <f t="shared" si="1"/>
-        <v>25</v>
-      </c>
-      <c r="N31" s="91"/>
-      <c r="O31" s="93" t="s">
-        <v>225</v>
-      </c>
-      <c r="P31" s="94" t="s">
-        <v>225</v>
-      </c>
-      <c r="Q31" s="94" t="s">
-        <v>225</v>
-      </c>
-      <c r="R31" s="74"/>
-      <c r="S31" s="94"/>
+        <v>139</v>
+      </c>
+      <c r="H31" s="61" t="s">
+        <v>159</v>
+      </c>
+      <c r="I31" s="61" t="s">
+        <v>284</v>
+      </c>
+      <c r="J31" s="61" t="s">
+        <v>239</v>
+      </c>
+      <c r="K31" s="68" t="s">
+        <v>193</v>
+      </c>
+      <c r="L31" s="111">
+        <v>3</v>
+      </c>
+      <c r="M31" s="111">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+      <c r="N31" s="61">
+        <v>100</v>
+      </c>
+      <c r="O31" s="69" t="s">
+        <v>223</v>
+      </c>
+      <c r="P31" s="70">
+        <v>6.9999999999999999E-4</v>
+      </c>
+      <c r="Q31" s="70">
+        <f t="shared" si="2"/>
+        <v>6.9999999999999993E-2</v>
+      </c>
+      <c r="R31" s="67"/>
+      <c r="S31" s="70"/>
     </row>
     <row r="32" spans="1:19" s="64" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="63"/>
       <c r="B32" s="37">
+        <f>ROW(B32) - ROW($B$9)</f>
+        <v>23</v>
+      </c>
+      <c r="C32" s="53" t="s">
+        <v>204</v>
+      </c>
+      <c r="D32" s="71" t="s">
+        <v>33</v>
+      </c>
+      <c r="E32" s="67" t="s">
+        <v>74</v>
+      </c>
+      <c r="F32" s="61" t="s">
+        <v>108</v>
+      </c>
+      <c r="G32" s="67" t="s">
+        <v>140</v>
+      </c>
+      <c r="H32" s="61" t="s">
+        <v>152</v>
+      </c>
+      <c r="I32" s="61" t="s">
+        <v>225</v>
+      </c>
+      <c r="J32" s="61" t="s">
+        <v>250</v>
+      </c>
+      <c r="K32" s="68" t="s">
+        <v>194</v>
+      </c>
+      <c r="L32" s="61">
+        <v>8</v>
+      </c>
+      <c r="M32" s="61">
         <f t="shared" si="0"/>
-        <v>23</v>
-      </c>
-      <c r="C32" s="52" t="s">
-        <v>204</v>
-      </c>
-      <c r="D32" s="72" t="s">
-        <v>32</v>
-      </c>
-      <c r="E32" s="45" t="s">
-        <v>73</v>
-      </c>
-      <c r="F32" s="45" t="s">
-        <v>107</v>
-      </c>
-      <c r="G32" s="73" t="s">
-        <v>139</v>
-      </c>
-      <c r="H32" s="45" t="s">
-        <v>159</v>
-      </c>
-      <c r="I32" s="45" t="s">
-        <v>284</v>
-      </c>
-      <c r="J32" s="45" t="s">
-        <v>239</v>
-      </c>
-      <c r="K32" s="58" t="s">
-        <v>193</v>
-      </c>
-      <c r="L32" s="59">
-        <v>3</v>
-      </c>
-      <c r="M32" s="59">
-        <f t="shared" si="1"/>
-        <v>15</v>
-      </c>
-      <c r="N32" s="45">
+        <v>40</v>
+      </c>
+      <c r="N32" s="61">
         <v>100</v>
       </c>
-      <c r="O32" s="62" t="s">
+      <c r="O32" s="69" t="s">
         <v>223</v>
       </c>
-      <c r="P32" s="47">
-        <v>6.9999999999999999E-4</v>
-      </c>
-      <c r="Q32" s="47">
+      <c r="P32" s="70">
+        <v>1.1000000000000001E-3</v>
+      </c>
+      <c r="Q32" s="70">
         <f t="shared" si="2"/>
-        <v>6.9999999999999993E-2</v>
-      </c>
-      <c r="R32" s="46"/>
-      <c r="S32" s="47"/>
+        <v>0.11</v>
+      </c>
+      <c r="R32" s="67"/>
+      <c r="S32" s="70"/>
     </row>
     <row r="33" spans="1:19" s="64" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="63"/>
       <c r="B33" s="37">
-        <f>ROW(B33) - ROW($B$9)</f>
+        <f t="shared" si="1"/>
         <v>24</v>
       </c>
       <c r="C33" s="53" t="s">
         <v>204</v>
       </c>
-      <c r="D33" s="71" t="s">
-        <v>33</v>
-      </c>
-      <c r="E33" s="67" t="s">
-        <v>74</v>
+      <c r="D33" s="110" t="s">
+        <v>34</v>
+      </c>
+      <c r="E33" s="61" t="s">
+        <v>75</v>
       </c>
       <c r="F33" s="61" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G33" s="67" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="H33" s="61" t="s">
         <v>152</v>
@@ -3797,17 +3844,17 @@
         <v>225</v>
       </c>
       <c r="J33" s="61" t="s">
-        <v>250</v>
+        <v>242</v>
       </c>
       <c r="K33" s="68" t="s">
-        <v>194</v>
-      </c>
-      <c r="L33" s="61">
-        <v>8</v>
-      </c>
-      <c r="M33" s="61">
-        <f t="shared" si="1"/>
-        <v>40</v>
+        <v>195</v>
+      </c>
+      <c r="L33" s="111">
+        <v>3</v>
+      </c>
+      <c r="M33" s="111">
+        <f t="shared" si="0"/>
+        <v>15</v>
       </c>
       <c r="N33" s="61">
         <v>100</v>
@@ -3816,91 +3863,91 @@
         <v>223</v>
       </c>
       <c r="P33" s="70">
-        <v>1.1000000000000001E-3</v>
+        <v>1.1999999999999999E-3</v>
       </c>
       <c r="Q33" s="70">
         <f t="shared" si="2"/>
-        <v>0.11</v>
+        <v>0.12</v>
       </c>
       <c r="R33" s="67"/>
       <c r="S33" s="70"/>
     </row>
-    <row r="34" spans="1:19" s="64" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:19" s="64" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="63"/>
       <c r="B34" s="37">
+        <f>ROW(B34) - ROW($B$9)</f>
+        <v>25</v>
+      </c>
+      <c r="C34" s="53" t="s">
+        <v>204</v>
+      </c>
+      <c r="D34" s="71" t="s">
+        <v>35</v>
+      </c>
+      <c r="E34" s="67" t="s">
+        <v>76</v>
+      </c>
+      <c r="F34" s="61" t="s">
+        <v>108</v>
+      </c>
+      <c r="G34" s="67" t="s">
+        <v>142</v>
+      </c>
+      <c r="H34" s="61" t="s">
+        <v>152</v>
+      </c>
+      <c r="I34" s="61" t="s">
+        <v>225</v>
+      </c>
+      <c r="J34" s="61" t="s">
+        <v>177</v>
+      </c>
+      <c r="K34" s="68" t="s">
+        <v>196</v>
+      </c>
+      <c r="L34" s="61">
+        <v>10</v>
+      </c>
+      <c r="M34" s="61">
         <f t="shared" si="0"/>
-        <v>25</v>
-      </c>
-      <c r="C34" s="52" t="s">
-        <v>204</v>
-      </c>
-      <c r="D34" s="72" t="s">
-        <v>34</v>
-      </c>
-      <c r="E34" s="45" t="s">
-        <v>75</v>
-      </c>
-      <c r="F34" s="45" t="s">
-        <v>107</v>
-      </c>
-      <c r="G34" s="46" t="s">
-        <v>141</v>
-      </c>
-      <c r="H34" s="45" t="s">
-        <v>152</v>
-      </c>
-      <c r="I34" s="45" t="s">
-        <v>225</v>
-      </c>
-      <c r="J34" s="45" t="s">
-        <v>242</v>
-      </c>
-      <c r="K34" s="58" t="s">
-        <v>195</v>
-      </c>
-      <c r="L34" s="59">
-        <v>3</v>
-      </c>
-      <c r="M34" s="59">
-        <f t="shared" si="1"/>
-        <v>15</v>
-      </c>
-      <c r="N34" s="45">
+        <v>50</v>
+      </c>
+      <c r="N34" s="61">
         <v>100</v>
       </c>
-      <c r="O34" s="62" t="s">
+      <c r="O34" s="69" t="s">
         <v>223</v>
       </c>
-      <c r="P34" s="47">
-        <v>1.1999999999999999E-3</v>
-      </c>
-      <c r="Q34" s="47">
+      <c r="P34" s="70">
+        <v>1.1000000000000001E-3</v>
+      </c>
+      <c r="Q34" s="70">
         <f t="shared" si="2"/>
-        <v>0.12</v>
-      </c>
-      <c r="R34" s="46"/>
-      <c r="S34" s="47"/>
+        <v>0.11</v>
+      </c>
+      <c r="R34" s="67"/>
+      <c r="S34" s="70"/>
     </row>
     <row r="35" spans="1:19" s="64" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="63"/>
       <c r="B35" s="37">
-        <f>ROW(B35) - ROW($B$9)</f>
+        <f t="shared" si="1"/>
         <v>26</v>
       </c>
       <c r="C35" s="53" t="s">
         <v>204</v>
       </c>
-      <c r="D35" s="71" t="s">
-        <v>35</v>
-      </c>
-      <c r="E35" s="67" t="s">
-        <v>76</v>
+      <c r="D35" s="110" t="s">
+        <v>36</v>
+      </c>
+      <c r="E35" s="61" t="s">
+        <v>77</v>
       </c>
       <c r="F35" s="61" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G35" s="67" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H35" s="61" t="s">
         <v>152</v>
@@ -3909,17 +3956,17 @@
         <v>225</v>
       </c>
       <c r="J35" s="61" t="s">
-        <v>177</v>
+        <v>243</v>
       </c>
       <c r="K35" s="68" t="s">
-        <v>196</v>
-      </c>
-      <c r="L35" s="61">
+        <v>197</v>
+      </c>
+      <c r="L35" s="111">
+        <v>2</v>
+      </c>
+      <c r="M35" s="111">
+        <f t="shared" si="0"/>
         <v>10</v>
-      </c>
-      <c r="M35" s="61">
-        <f t="shared" si="1"/>
-        <v>50</v>
       </c>
       <c r="N35" s="61">
         <v>100</v>
@@ -3937,63 +3984,63 @@
       <c r="R35" s="67"/>
       <c r="S35" s="70"/>
     </row>
-    <row r="36" spans="1:19" s="64" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:19" s="64" customFormat="1" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="63"/>
       <c r="B36" s="37">
+        <f>ROW(B36) - ROW($B$9)</f>
+        <v>27</v>
+      </c>
+      <c r="C36" s="53" t="s">
+        <v>204</v>
+      </c>
+      <c r="D36" s="71" t="s">
+        <v>259</v>
+      </c>
+      <c r="E36" s="67" t="s">
+        <v>78</v>
+      </c>
+      <c r="F36" s="61" t="s">
+        <v>109</v>
+      </c>
+      <c r="G36" s="67" t="s">
+        <v>144</v>
+      </c>
+      <c r="H36" s="61" t="s">
+        <v>152</v>
+      </c>
+      <c r="I36" s="61" t="s">
+        <v>225</v>
+      </c>
+      <c r="J36" s="61" t="s">
+        <v>178</v>
+      </c>
+      <c r="K36" s="68" t="s">
+        <v>198</v>
+      </c>
+      <c r="L36" s="61">
+        <v>17</v>
+      </c>
+      <c r="M36" s="61">
         <f t="shared" si="0"/>
-        <v>27</v>
-      </c>
-      <c r="C36" s="52" t="s">
-        <v>204</v>
-      </c>
-      <c r="D36" s="72" t="s">
-        <v>36</v>
-      </c>
-      <c r="E36" s="45" t="s">
-        <v>77</v>
-      </c>
-      <c r="F36" s="45" t="s">
-        <v>107</v>
-      </c>
-      <c r="G36" s="46" t="s">
-        <v>143</v>
-      </c>
-      <c r="H36" s="45" t="s">
-        <v>152</v>
-      </c>
-      <c r="I36" s="45" t="s">
-        <v>225</v>
-      </c>
-      <c r="J36" s="45" t="s">
-        <v>243</v>
-      </c>
-      <c r="K36" s="58" t="s">
-        <v>197</v>
-      </c>
-      <c r="L36" s="59">
-        <v>2</v>
-      </c>
-      <c r="M36" s="59">
-        <f t="shared" si="1"/>
-        <v>10</v>
-      </c>
-      <c r="N36" s="45">
+        <v>85</v>
+      </c>
+      <c r="N36" s="61">
         <v>100</v>
       </c>
-      <c r="O36" s="62" t="s">
+      <c r="O36" s="69" t="s">
         <v>223</v>
       </c>
-      <c r="P36" s="47">
-        <v>1.1000000000000001E-3</v>
-      </c>
-      <c r="Q36" s="47">
+      <c r="P36" s="70">
+        <v>5.9999999999999995E-4</v>
+      </c>
+      <c r="Q36" s="70">
         <f t="shared" si="2"/>
-        <v>0.11</v>
-      </c>
-      <c r="R36" s="46"/>
-      <c r="S36" s="47"/>
-    </row>
-    <row r="37" spans="1:19" s="64" customFormat="1" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>0.06</v>
+      </c>
+      <c r="R36" s="67"/>
+      <c r="S36" s="70"/>
+    </row>
+    <row r="37" spans="1:19" s="64" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="63"/>
       <c r="B37" s="37">
         <f>ROW(B37) - ROW($B$9)</f>
@@ -4002,17 +4049,17 @@
       <c r="C37" s="53" t="s">
         <v>204</v>
       </c>
-      <c r="D37" s="71" t="s">
-        <v>259</v>
-      </c>
-      <c r="E37" s="67" t="s">
-        <v>78</v>
+      <c r="D37" s="110" t="s">
+        <v>37</v>
+      </c>
+      <c r="E37" s="61" t="s">
+        <v>79</v>
       </c>
       <c r="F37" s="61" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G37" s="67" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="H37" s="61" t="s">
         <v>152</v>
@@ -4021,17 +4068,17 @@
         <v>225</v>
       </c>
       <c r="J37" s="61" t="s">
-        <v>178</v>
+        <v>251</v>
       </c>
       <c r="K37" s="68" t="s">
-        <v>198</v>
-      </c>
-      <c r="L37" s="61">
-        <v>17</v>
-      </c>
-      <c r="M37" s="61">
-        <f t="shared" si="1"/>
-        <v>85</v>
+        <v>199</v>
+      </c>
+      <c r="L37" s="111">
+        <v>4</v>
+      </c>
+      <c r="M37" s="111">
+        <f t="shared" si="0"/>
+        <v>20</v>
       </c>
       <c r="N37" s="61">
         <v>100</v>
@@ -4040,541 +4087,543 @@
         <v>223</v>
       </c>
       <c r="P37" s="70">
-        <v>5.9999999999999995E-4</v>
+        <v>1.2999999999999999E-3</v>
       </c>
       <c r="Q37" s="70">
         <f t="shared" si="2"/>
-        <v>0.06</v>
+        <v>0.13</v>
       </c>
       <c r="R37" s="67"/>
       <c r="S37" s="70"/>
     </row>
-    <row r="38" spans="1:19" s="64" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:19" s="64" customFormat="1" ht="216.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="63"/>
       <c r="B38" s="37">
-        <f>ROW(B38) - ROW($B$9)</f>
+        <f t="shared" si="1"/>
         <v>29</v>
       </c>
-      <c r="C38" s="52" t="s">
-        <v>204</v>
-      </c>
-      <c r="D38" s="72" t="s">
-        <v>37</v>
-      </c>
-      <c r="E38" s="45" t="s">
-        <v>79</v>
-      </c>
-      <c r="F38" s="45" t="s">
-        <v>108</v>
-      </c>
-      <c r="G38" s="46" t="s">
-        <v>145</v>
-      </c>
-      <c r="H38" s="45" t="s">
-        <v>152</v>
-      </c>
-      <c r="I38" s="45" t="s">
-        <v>225</v>
-      </c>
-      <c r="J38" s="45" t="s">
-        <v>251</v>
-      </c>
-      <c r="K38" s="58" t="s">
-        <v>199</v>
-      </c>
-      <c r="L38" s="59">
-        <v>4</v>
-      </c>
-      <c r="M38" s="59">
-        <f t="shared" si="1"/>
-        <v>20</v>
-      </c>
-      <c r="N38" s="45">
-        <v>100</v>
-      </c>
-      <c r="O38" s="62" t="s">
-        <v>223</v>
-      </c>
-      <c r="P38" s="47">
-        <v>1.2999999999999999E-3</v>
-      </c>
-      <c r="Q38" s="47">
-        <f t="shared" si="2"/>
-        <v>0.13</v>
-      </c>
-      <c r="R38" s="46"/>
-      <c r="S38" s="47"/>
-    </row>
-    <row r="39" spans="1:19" s="64" customFormat="1" ht="216.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C38" s="53" t="s">
+        <v>205</v>
+      </c>
+      <c r="D38" s="90" t="s">
+        <v>38</v>
+      </c>
+      <c r="E38" s="74" t="s">
+        <v>80</v>
+      </c>
+      <c r="F38" s="91" t="s">
+        <v>230</v>
+      </c>
+      <c r="G38" s="74" t="s">
+        <v>110</v>
+      </c>
+      <c r="H38" s="91" t="s">
+        <v>225</v>
+      </c>
+      <c r="I38" s="91" t="s">
+        <v>225</v>
+      </c>
+      <c r="J38" s="91" t="s">
+        <v>225</v>
+      </c>
+      <c r="K38" s="92" t="s">
+        <v>225</v>
+      </c>
+      <c r="L38" s="91">
+        <v>106</v>
+      </c>
+      <c r="M38" s="91">
+        <f t="shared" si="0"/>
+        <v>530</v>
+      </c>
+      <c r="N38" s="91"/>
+      <c r="O38" s="93" t="s">
+        <v>225</v>
+      </c>
+      <c r="P38" s="94" t="s">
+        <v>225</v>
+      </c>
+      <c r="Q38" s="94" t="s">
+        <v>225</v>
+      </c>
+      <c r="R38" s="74"/>
+      <c r="S38" s="94"/>
+    </row>
+    <row r="39" spans="1:19" s="64" customFormat="1" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="63"/>
       <c r="B39" s="37">
+        <f>ROW(B39) - ROW($B$9)</f>
+        <v>30</v>
+      </c>
+      <c r="C39" s="53" t="s">
+        <v>206</v>
+      </c>
+      <c r="D39" s="110" t="s">
+        <v>39</v>
+      </c>
+      <c r="E39" s="61" t="s">
+        <v>81</v>
+      </c>
+      <c r="F39" s="61" t="s">
+        <v>230</v>
+      </c>
+      <c r="G39" s="67" t="s">
+        <v>111</v>
+      </c>
+      <c r="H39" s="61" t="s">
+        <v>160</v>
+      </c>
+      <c r="I39" s="61" t="s">
+        <v>225</v>
+      </c>
+      <c r="J39" s="61" t="s">
+        <v>275</v>
+      </c>
+      <c r="K39" s="68" t="s">
+        <v>225</v>
+      </c>
+      <c r="L39" s="111">
+        <v>1</v>
+      </c>
+      <c r="M39" s="111">
         <f t="shared" si="0"/>
-        <v>30</v>
-      </c>
-      <c r="C39" s="53" t="s">
-        <v>205</v>
-      </c>
-      <c r="D39" s="90" t="s">
-        <v>38</v>
-      </c>
-      <c r="E39" s="74" t="s">
-        <v>80</v>
-      </c>
-      <c r="F39" s="91" t="s">
-        <v>230</v>
-      </c>
-      <c r="G39" s="74" t="s">
-        <v>110</v>
-      </c>
-      <c r="H39" s="91" t="s">
-        <v>225</v>
-      </c>
-      <c r="I39" s="91" t="s">
-        <v>225</v>
-      </c>
-      <c r="J39" s="91" t="s">
-        <v>225</v>
-      </c>
-      <c r="K39" s="92" t="s">
-        <v>225</v>
-      </c>
-      <c r="L39" s="91">
-        <v>106</v>
-      </c>
-      <c r="M39" s="91">
-        <f t="shared" si="1"/>
-        <v>530</v>
-      </c>
-      <c r="N39" s="91"/>
-      <c r="O39" s="93" t="s">
-        <v>225</v>
-      </c>
-      <c r="P39" s="94" t="s">
-        <v>225</v>
-      </c>
-      <c r="Q39" s="94" t="s">
-        <v>225</v>
-      </c>
-      <c r="R39" s="74"/>
-      <c r="S39" s="94"/>
-    </row>
-    <row r="40" spans="1:19" s="64" customFormat="1" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>5</v>
+      </c>
+      <c r="N39" s="61">
+        <v>10</v>
+      </c>
+      <c r="O39" s="69" t="s">
+        <v>223</v>
+      </c>
+      <c r="P39" s="70">
+        <v>5.7599999999999998E-2</v>
+      </c>
+      <c r="Q39" s="70">
+        <f t="shared" si="2"/>
+        <v>0.57599999999999996</v>
+      </c>
+      <c r="R39" s="95"/>
+      <c r="S39" s="70"/>
+    </row>
+    <row r="40" spans="1:19" s="64" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="63"/>
       <c r="B40" s="37">
-        <f>ROW(B40) - ROW($B$9)</f>
+        <f t="shared" si="1"/>
         <v>31</v>
       </c>
-      <c r="C40" s="52" t="s">
-        <v>206</v>
-      </c>
-      <c r="D40" s="72" t="s">
-        <v>39</v>
-      </c>
-      <c r="E40" s="45" t="s">
-        <v>81</v>
-      </c>
-      <c r="F40" s="45" t="s">
+      <c r="C40" s="53" t="s">
+        <v>10</v>
+      </c>
+      <c r="D40" s="71" t="s">
+        <v>40</v>
+      </c>
+      <c r="E40" s="67" t="s">
+        <v>82</v>
+      </c>
+      <c r="F40" s="61" t="s">
         <v>230</v>
       </c>
-      <c r="G40" s="46" t="s">
-        <v>111</v>
-      </c>
-      <c r="H40" s="45" t="s">
-        <v>160</v>
-      </c>
-      <c r="I40" s="45" t="s">
-        <v>225</v>
-      </c>
-      <c r="J40" s="45" t="s">
-        <v>275</v>
-      </c>
-      <c r="K40" s="58" t="s">
-        <v>225</v>
-      </c>
-      <c r="L40" s="59">
+      <c r="G40" s="67" t="s">
+        <v>112</v>
+      </c>
+      <c r="H40" s="61" t="s">
+        <v>163</v>
+      </c>
+      <c r="I40" s="61" t="s">
+        <v>225</v>
+      </c>
+      <c r="J40" s="61" t="s">
+        <v>179</v>
+      </c>
+      <c r="K40" s="68" t="s">
+        <v>225</v>
+      </c>
+      <c r="L40" s="61">
         <v>1</v>
       </c>
-      <c r="M40" s="59">
-        <f t="shared" si="1"/>
+      <c r="M40" s="61">
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N40" s="45">
-        <v>10</v>
-      </c>
-      <c r="O40" s="62" t="s">
+      <c r="N40" s="61">
+        <v>6</v>
+      </c>
+      <c r="O40" s="69" t="s">
         <v>223</v>
       </c>
-      <c r="P40" s="47">
-        <v>5.7599999999999998E-2</v>
-      </c>
-      <c r="Q40" s="47">
+      <c r="P40" s="70">
+        <v>4.1506999999999996</v>
+      </c>
+      <c r="Q40" s="70">
         <f t="shared" si="2"/>
-        <v>0.57599999999999996</v>
-      </c>
-      <c r="R40" s="89"/>
-      <c r="S40" s="47"/>
+        <v>24.904199999999996</v>
+      </c>
+      <c r="R40" s="67"/>
+      <c r="S40" s="70"/>
     </row>
     <row r="41" spans="1:19" s="64" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="63"/>
       <c r="B41" s="37">
+        <f>ROW(B41) - ROW($B$9)</f>
+        <v>32</v>
+      </c>
+      <c r="C41" s="53" t="s">
+        <v>11</v>
+      </c>
+      <c r="D41" s="110" t="s">
+        <v>41</v>
+      </c>
+      <c r="E41" s="61" t="s">
+        <v>83</v>
+      </c>
+      <c r="F41" s="61" t="s">
+        <v>113</v>
+      </c>
+      <c r="G41" s="67" t="s">
+        <v>146</v>
+      </c>
+      <c r="H41" s="61" t="s">
+        <v>158</v>
+      </c>
+      <c r="I41" s="61" t="s">
+        <v>225</v>
+      </c>
+      <c r="J41" s="61" t="s">
+        <v>180</v>
+      </c>
+      <c r="K41" s="68" t="s">
+        <v>225</v>
+      </c>
+      <c r="L41" s="111">
+        <v>8</v>
+      </c>
+      <c r="M41" s="111">
         <f t="shared" si="0"/>
-        <v>32</v>
-      </c>
-      <c r="C41" s="53" t="s">
-        <v>10</v>
-      </c>
-      <c r="D41" s="71" t="s">
         <v>40</v>
       </c>
-      <c r="E41" s="67" t="s">
-        <v>82</v>
-      </c>
-      <c r="F41" s="61" t="s">
-        <v>230</v>
-      </c>
-      <c r="G41" s="67" t="s">
-        <v>112</v>
-      </c>
-      <c r="H41" s="61" t="s">
-        <v>163</v>
-      </c>
-      <c r="I41" s="61" t="s">
-        <v>225</v>
-      </c>
-      <c r="J41" s="61" t="s">
-        <v>179</v>
-      </c>
-      <c r="K41" s="68" t="s">
-        <v>225</v>
-      </c>
-      <c r="L41" s="61">
-        <v>1</v>
-      </c>
-      <c r="M41" s="61">
-        <f t="shared" si="1"/>
-        <v>5</v>
-      </c>
       <c r="N41" s="61">
-        <v>6</v>
+        <v>42</v>
       </c>
       <c r="O41" s="69" t="s">
         <v>223</v>
       </c>
       <c r="P41" s="70">
-        <v>4.1506999999999996</v>
+        <v>4.2987000000000002</v>
       </c>
       <c r="Q41" s="70">
         <f t="shared" si="2"/>
-        <v>24.904199999999996</v>
+        <v>180.5454</v>
       </c>
       <c r="R41" s="67"/>
       <c r="S41" s="70"/>
     </row>
-    <row r="42" spans="1:19" s="64" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:19" s="64" customFormat="1" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="63"/>
       <c r="B42" s="37">
-        <f>ROW(B42) - ROW($B$9)</f>
+        <f t="shared" si="1"/>
         <v>33</v>
       </c>
-      <c r="C42" s="52" t="s">
+      <c r="C42" s="53" t="s">
         <v>11</v>
       </c>
-      <c r="D42" s="72" t="s">
-        <v>41</v>
-      </c>
-      <c r="E42" s="45" t="s">
-        <v>83</v>
-      </c>
-      <c r="F42" s="45" t="s">
-        <v>113</v>
-      </c>
-      <c r="G42" s="46" t="s">
-        <v>146</v>
-      </c>
-      <c r="H42" s="45" t="s">
-        <v>158</v>
-      </c>
-      <c r="I42" s="45" t="s">
-        <v>225</v>
-      </c>
-      <c r="J42" s="45" t="s">
-        <v>180</v>
-      </c>
-      <c r="K42" s="58" t="s">
-        <v>225</v>
-      </c>
-      <c r="L42" s="59">
-        <v>8</v>
-      </c>
-      <c r="M42" s="59">
-        <f t="shared" si="1"/>
-        <v>40</v>
-      </c>
-      <c r="N42" s="45">
+      <c r="D42" s="71" t="s">
         <v>42</v>
       </c>
-      <c r="O42" s="62" t="s">
+      <c r="E42" s="67" t="s">
+        <v>84</v>
+      </c>
+      <c r="F42" s="61" t="s">
+        <v>114</v>
+      </c>
+      <c r="G42" s="67" t="s">
+        <v>147</v>
+      </c>
+      <c r="H42" s="61" t="s">
+        <v>164</v>
+      </c>
+      <c r="I42" s="61" t="s">
+        <v>225</v>
+      </c>
+      <c r="J42" s="61" t="s">
+        <v>252</v>
+      </c>
+      <c r="K42" s="68" t="s">
+        <v>225</v>
+      </c>
+      <c r="L42" s="61">
+        <v>1</v>
+      </c>
+      <c r="M42" s="61">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="N42" s="61">
+        <v>6</v>
+      </c>
+      <c r="O42" s="69" t="s">
         <v>223</v>
       </c>
-      <c r="P42" s="47">
-        <v>4.2987000000000002</v>
-      </c>
-      <c r="Q42" s="47">
+      <c r="P42" s="70">
+        <v>0.51070000000000004</v>
+      </c>
+      <c r="Q42" s="70">
         <f t="shared" si="2"/>
-        <v>180.5454</v>
-      </c>
-      <c r="R42" s="46"/>
-      <c r="S42" s="47"/>
-    </row>
-    <row r="43" spans="1:19" s="64" customFormat="1" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>3.0642000000000005</v>
+      </c>
+      <c r="R42" s="67"/>
+      <c r="S42" s="70"/>
+    </row>
+    <row r="43" spans="1:19" s="64" customFormat="1" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="63"/>
       <c r="B43" s="37">
-        <f t="shared" si="0"/>
+        <f>ROW(B43) - ROW($B$9)</f>
         <v>34</v>
       </c>
       <c r="C43" s="53" t="s">
         <v>11</v>
       </c>
-      <c r="D43" s="71" t="s">
-        <v>42</v>
-      </c>
-      <c r="E43" s="67" t="s">
-        <v>84</v>
+      <c r="D43" s="110" t="s">
+        <v>43</v>
+      </c>
+      <c r="E43" s="61" t="s">
+        <v>85</v>
       </c>
       <c r="F43" s="61" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="G43" s="67" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="H43" s="61" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="I43" s="61" t="s">
         <v>225</v>
       </c>
       <c r="J43" s="61" t="s">
-        <v>252</v>
+        <v>225</v>
       </c>
       <c r="K43" s="68" t="s">
         <v>225</v>
       </c>
-      <c r="L43" s="61">
+      <c r="L43" s="111">
         <v>1</v>
       </c>
-      <c r="M43" s="61">
-        <f t="shared" si="1"/>
+      <c r="M43" s="111">
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="N43" s="61">
         <v>6</v>
       </c>
       <c r="O43" s="69" t="s">
-        <v>223</v>
+        <v>231</v>
       </c>
       <c r="P43" s="70">
-        <v>0.51070000000000004</v>
+        <v>12.6</v>
       </c>
       <c r="Q43" s="70">
         <f t="shared" si="2"/>
-        <v>3.0642000000000005</v>
-      </c>
-      <c r="R43" s="67"/>
+        <v>75.599999999999994</v>
+      </c>
+      <c r="R43" s="95" t="s">
+        <v>269</v>
+      </c>
       <c r="S43" s="70"/>
     </row>
-    <row r="44" spans="1:19" s="64" customFormat="1" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:19" s="64" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="63"/>
       <c r="B44" s="37">
-        <f>ROW(B44) - ROW($B$9)</f>
+        <f t="shared" si="1"/>
         <v>35</v>
       </c>
-      <c r="C44" s="52" t="s">
+      <c r="C44" s="53" t="s">
         <v>11</v>
       </c>
-      <c r="D44" s="72" t="s">
-        <v>43</v>
-      </c>
-      <c r="E44" s="45" t="s">
-        <v>85</v>
-      </c>
-      <c r="F44" s="45" t="s">
-        <v>115</v>
-      </c>
-      <c r="G44" s="46" t="s">
-        <v>148</v>
-      </c>
-      <c r="H44" s="45" t="s">
+      <c r="D44" s="71" t="s">
+        <v>44</v>
+      </c>
+      <c r="E44" s="67" t="s">
+        <v>86</v>
+      </c>
+      <c r="F44" s="61" t="s">
+        <v>240</v>
+      </c>
+      <c r="G44" s="67" t="s">
+        <v>116</v>
+      </c>
+      <c r="H44" s="61" t="s">
         <v>158</v>
       </c>
-      <c r="I44" s="45" t="s">
-        <v>225</v>
-      </c>
-      <c r="J44" s="45" t="s">
-        <v>225</v>
-      </c>
-      <c r="K44" s="58" t="s">
-        <v>225</v>
-      </c>
-      <c r="L44" s="59">
-        <v>1</v>
-      </c>
-      <c r="M44" s="59">
-        <f t="shared" si="1"/>
-        <v>5</v>
-      </c>
-      <c r="N44" s="45">
-        <v>6</v>
-      </c>
-      <c r="O44" s="62" t="s">
-        <v>231</v>
-      </c>
-      <c r="P44" s="47">
-        <v>12.6</v>
-      </c>
-      <c r="Q44" s="47">
+      <c r="I44" s="61" t="s">
+        <v>225</v>
+      </c>
+      <c r="J44" s="61" t="s">
+        <v>233</v>
+      </c>
+      <c r="K44" s="68" t="s">
+        <v>225</v>
+      </c>
+      <c r="L44" s="61">
+        <v>2</v>
+      </c>
+      <c r="M44" s="61">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="N44" s="61">
+        <v>11</v>
+      </c>
+      <c r="O44" s="69" t="s">
+        <v>223</v>
+      </c>
+      <c r="P44" s="70">
+        <v>3.8660000000000001</v>
+      </c>
+      <c r="Q44" s="70">
         <f t="shared" si="2"/>
-        <v>75.599999999999994</v>
-      </c>
-      <c r="R44" s="89" t="s">
-        <v>269</v>
-      </c>
-      <c r="S44" s="47"/>
-    </row>
-    <row r="45" spans="1:19" s="64" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>42.526000000000003</v>
+      </c>
+      <c r="R44" s="67"/>
+      <c r="S44" s="70"/>
+    </row>
+    <row r="45" spans="1:19" s="64" customFormat="1" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="63"/>
       <c r="B45" s="37">
-        <f t="shared" si="0"/>
+        <f>ROW(B45) - ROW($B$9)</f>
         <v>36</v>
       </c>
       <c r="C45" s="53" t="s">
         <v>11</v>
       </c>
-      <c r="D45" s="71" t="s">
-        <v>44</v>
-      </c>
-      <c r="E45" s="67" t="s">
-        <v>86</v>
+      <c r="D45" s="110" t="s">
+        <v>45</v>
+      </c>
+      <c r="E45" s="61" t="s">
+        <v>87</v>
       </c>
       <c r="F45" s="61" t="s">
-        <v>240</v>
-      </c>
-      <c r="G45" s="67" t="s">
-        <v>116</v>
+        <v>241</v>
+      </c>
+      <c r="G45" s="112" t="s">
+        <v>117</v>
       </c>
       <c r="H45" s="61" t="s">
-        <v>158</v>
+        <v>165</v>
       </c>
       <c r="I45" s="61" t="s">
         <v>225</v>
       </c>
       <c r="J45" s="61" t="s">
-        <v>233</v>
+        <v>225</v>
       </c>
       <c r="K45" s="68" t="s">
         <v>225</v>
       </c>
-      <c r="L45" s="61">
-        <v>2</v>
-      </c>
-      <c r="M45" s="61">
-        <f t="shared" si="1"/>
+      <c r="L45" s="111">
+        <v>1</v>
+      </c>
+      <c r="M45" s="111">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="N45" s="61">
         <v>10</v>
       </c>
-      <c r="N45" s="61">
-        <v>11</v>
-      </c>
       <c r="O45" s="69" t="s">
-        <v>223</v>
+        <v>276</v>
       </c>
       <c r="P45" s="70">
-        <v>3.8660000000000001</v>
+        <v>6.3399999999999998E-2</v>
       </c>
       <c r="Q45" s="70">
         <f t="shared" si="2"/>
-        <v>42.526000000000003</v>
+        <v>0.63400000000000001</v>
       </c>
       <c r="R45" s="67"/>
       <c r="S45" s="70"/>
     </row>
-    <row r="46" spans="1:19" s="64" customFormat="1" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:19" s="64" customFormat="1" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="63"/>
       <c r="B46" s="37">
-        <f>ROW(B46) - ROW($B$9)</f>
+        <f t="shared" si="1"/>
         <v>37</v>
       </c>
-      <c r="C46" s="52" t="s">
+      <c r="C46" s="53" t="s">
         <v>11</v>
       </c>
-      <c r="D46" s="72" t="s">
-        <v>45</v>
-      </c>
-      <c r="E46" s="45" t="s">
-        <v>87</v>
-      </c>
-      <c r="F46" s="45" t="s">
-        <v>241</v>
-      </c>
-      <c r="G46" s="98" t="s">
-        <v>117</v>
-      </c>
-      <c r="H46" s="45" t="s">
-        <v>165</v>
-      </c>
-      <c r="I46" s="45" t="s">
-        <v>225</v>
-      </c>
-      <c r="J46" s="45" t="s">
-        <v>225</v>
-      </c>
-      <c r="K46" s="58" t="s">
-        <v>225</v>
-      </c>
-      <c r="L46" s="59">
+      <c r="D46" s="71" t="s">
+        <v>46</v>
+      </c>
+      <c r="E46" s="67" t="s">
+        <v>88</v>
+      </c>
+      <c r="F46" s="61" t="s">
+        <v>118</v>
+      </c>
+      <c r="G46" s="67" t="s">
+        <v>149</v>
+      </c>
+      <c r="H46" s="61" t="s">
+        <v>158</v>
+      </c>
+      <c r="I46" s="61" t="s">
+        <v>225</v>
+      </c>
+      <c r="J46" s="61" t="s">
+        <v>225</v>
+      </c>
+      <c r="K46" s="68" t="s">
+        <v>225</v>
+      </c>
+      <c r="L46" s="61">
         <v>1</v>
       </c>
-      <c r="M46" s="59">
-        <f t="shared" si="1"/>
+      <c r="M46" s="61">
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N46" s="45">
-        <v>10</v>
-      </c>
-      <c r="O46" s="62" t="s">
-        <v>276</v>
-      </c>
-      <c r="P46" s="47">
-        <v>6.3399999999999998E-2</v>
-      </c>
-      <c r="Q46" s="47">
+      <c r="N46" s="61">
+        <v>6</v>
+      </c>
+      <c r="O46" s="69" t="s">
+        <v>231</v>
+      </c>
+      <c r="P46" s="70">
+        <v>7.3</v>
+      </c>
+      <c r="Q46" s="70">
         <f t="shared" si="2"/>
-        <v>0.63400000000000001</v>
-      </c>
-      <c r="R46" s="46"/>
-      <c r="S46" s="47"/>
+        <v>43.8</v>
+      </c>
+      <c r="R46" s="95" t="s">
+        <v>269</v>
+      </c>
+      <c r="S46" s="70"/>
     </row>
     <row r="47" spans="1:19" s="64" customFormat="1" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A47" s="63"/>
       <c r="B47" s="37">
-        <f t="shared" si="0"/>
+        <f>ROW(B47) - ROW($B$9)</f>
         <v>38</v>
       </c>
       <c r="C47" s="53" t="s">
         <v>11</v>
       </c>
-      <c r="D47" s="71" t="s">
-        <v>46</v>
-      </c>
-      <c r="E47" s="67" t="s">
-        <v>88</v>
+      <c r="D47" s="110" t="s">
+        <v>47</v>
+      </c>
+      <c r="E47" s="61" t="s">
+        <v>89</v>
       </c>
       <c r="F47" s="61" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G47" s="67" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="H47" s="61" t="s">
-        <v>158</v>
+        <v>166</v>
       </c>
       <c r="I47" s="61" t="s">
         <v>225</v>
@@ -4585,300 +4634,241 @@
       <c r="K47" s="68" t="s">
         <v>225</v>
       </c>
-      <c r="L47" s="61">
-        <v>1</v>
-      </c>
-      <c r="M47" s="61">
-        <f t="shared" si="1"/>
-        <v>5</v>
+      <c r="L47" s="111">
+        <v>4</v>
+      </c>
+      <c r="M47" s="111">
+        <f t="shared" si="0"/>
+        <v>20</v>
       </c>
       <c r="N47" s="61">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="O47" s="69" t="s">
         <v>231</v>
       </c>
       <c r="P47" s="70">
-        <v>7.3</v>
+        <v>4.2</v>
       </c>
       <c r="Q47" s="70">
         <f t="shared" si="2"/>
-        <v>43.8</v>
+        <v>88.2</v>
       </c>
       <c r="R47" s="95" t="s">
         <v>269</v>
       </c>
       <c r="S47" s="70"/>
     </row>
-    <row r="48" spans="1:19" s="64" customFormat="1" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:19" s="64" customFormat="1" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A48" s="63"/>
       <c r="B48" s="37">
-        <f>ROW(B48) - ROW($B$9)</f>
+        <f t="shared" si="1"/>
         <v>39</v>
       </c>
-      <c r="C48" s="52" t="s">
-        <v>11</v>
-      </c>
-      <c r="D48" s="72" t="s">
-        <v>47</v>
-      </c>
-      <c r="E48" s="45" t="s">
-        <v>89</v>
-      </c>
-      <c r="F48" s="45" t="s">
-        <v>119</v>
-      </c>
-      <c r="G48" s="46" t="s">
-        <v>150</v>
-      </c>
-      <c r="H48" s="45" t="s">
-        <v>166</v>
-      </c>
-      <c r="I48" s="45" t="s">
-        <v>225</v>
-      </c>
-      <c r="J48" s="45" t="s">
-        <v>225</v>
-      </c>
-      <c r="K48" s="58" t="s">
-        <v>225</v>
-      </c>
-      <c r="L48" s="59">
-        <v>4</v>
-      </c>
-      <c r="M48" s="59">
-        <f t="shared" si="1"/>
-        <v>20</v>
-      </c>
-      <c r="N48" s="45">
-        <v>21</v>
-      </c>
-      <c r="O48" s="62" t="s">
-        <v>231</v>
-      </c>
-      <c r="P48" s="47">
-        <v>4.2</v>
-      </c>
-      <c r="Q48" s="47">
+      <c r="C48" s="53" t="s">
+        <v>207</v>
+      </c>
+      <c r="D48" s="71" t="s">
+        <v>48</v>
+      </c>
+      <c r="E48" s="67" t="s">
+        <v>90</v>
+      </c>
+      <c r="F48" s="61" t="s">
+        <v>230</v>
+      </c>
+      <c r="G48" s="67" t="s">
+        <v>120</v>
+      </c>
+      <c r="H48" s="61" t="s">
+        <v>167</v>
+      </c>
+      <c r="I48" s="61" t="s">
+        <v>225</v>
+      </c>
+      <c r="J48" s="61" t="s">
+        <v>234</v>
+      </c>
+      <c r="K48" s="68" t="s">
+        <v>235</v>
+      </c>
+      <c r="L48" s="61">
+        <v>1</v>
+      </c>
+      <c r="M48" s="61">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="N48" s="61">
+        <v>6</v>
+      </c>
+      <c r="O48" s="69" t="s">
+        <v>223</v>
+      </c>
+      <c r="P48" s="70">
+        <v>0.23039999999999999</v>
+      </c>
+      <c r="Q48" s="70">
         <f t="shared" si="2"/>
-        <v>88.2</v>
-      </c>
-      <c r="R48" s="89" t="s">
-        <v>269</v>
-      </c>
-      <c r="S48" s="47"/>
+        <v>1.3824000000000001</v>
+      </c>
+      <c r="R48" s="67"/>
+      <c r="S48" s="70"/>
     </row>
     <row r="49" spans="1:19" s="64" customFormat="1" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A49" s="63"/>
       <c r="B49" s="37">
-        <f t="shared" si="0"/>
+        <f>ROW(B49) - ROW($B$9)</f>
         <v>40</v>
       </c>
       <c r="C49" s="53" t="s">
         <v>207</v>
       </c>
-      <c r="D49" s="71" t="s">
-        <v>48</v>
-      </c>
-      <c r="E49" s="67" t="s">
-        <v>90</v>
+      <c r="D49" s="110" t="s">
+        <v>49</v>
+      </c>
+      <c r="E49" s="61" t="s">
+        <v>91</v>
       </c>
       <c r="F49" s="61" t="s">
         <v>230</v>
       </c>
       <c r="G49" s="67" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="H49" s="61" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="I49" s="61" t="s">
         <v>225</v>
       </c>
       <c r="J49" s="61" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="K49" s="68" t="s">
-        <v>235</v>
-      </c>
-      <c r="L49" s="61">
-        <v>1</v>
-      </c>
-      <c r="M49" s="61">
-        <f t="shared" si="1"/>
-        <v>5</v>
+        <v>237</v>
+      </c>
+      <c r="L49" s="113">
+        <v>2</v>
+      </c>
+      <c r="M49" s="113">
+        <f t="shared" si="0"/>
+        <v>10</v>
       </c>
       <c r="N49" s="61">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="O49" s="69" t="s">
         <v>223</v>
       </c>
       <c r="P49" s="70">
-        <v>0.23039999999999999</v>
+        <v>7.6899999999999996E-2</v>
       </c>
       <c r="Q49" s="70">
         <f t="shared" si="2"/>
-        <v>1.3824000000000001</v>
+        <v>1.1535</v>
       </c>
       <c r="R49" s="67"/>
       <c r="S49" s="70"/>
     </row>
-    <row r="50" spans="1:19" s="64" customFormat="1" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="63"/>
-      <c r="B50" s="37">
-        <f>ROW(B50) - ROW($B$9)</f>
-        <v>41</v>
-      </c>
-      <c r="C50" s="52" t="s">
-        <v>207</v>
-      </c>
-      <c r="D50" s="72" t="s">
-        <v>49</v>
-      </c>
-      <c r="E50" s="45" t="s">
-        <v>91</v>
-      </c>
-      <c r="F50" s="45" t="s">
-        <v>230</v>
-      </c>
-      <c r="G50" s="46" t="s">
-        <v>121</v>
-      </c>
-      <c r="H50" s="45" t="s">
-        <v>168</v>
-      </c>
-      <c r="I50" s="45" t="s">
-        <v>225</v>
-      </c>
-      <c r="J50" s="45" t="s">
-        <v>236</v>
-      </c>
-      <c r="K50" s="58" t="s">
-        <v>237</v>
-      </c>
-      <c r="L50" s="75">
-        <v>2</v>
-      </c>
-      <c r="M50" s="75">
-        <f t="shared" si="1"/>
-        <v>10</v>
-      </c>
-      <c r="N50" s="45">
-        <v>15</v>
-      </c>
-      <c r="O50" s="62" t="s">
-        <v>223</v>
-      </c>
-      <c r="P50" s="47">
-        <v>7.6899999999999996E-2</v>
-      </c>
-      <c r="Q50" s="47">
-        <f t="shared" si="2"/>
-        <v>1.1535</v>
-      </c>
-      <c r="R50" s="46"/>
-      <c r="S50" s="47"/>
+    <row r="50" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A50" s="1"/>
+      <c r="B50" s="32"/>
+      <c r="C50" s="43"/>
+      <c r="D50" s="33"/>
+      <c r="E50" s="34"/>
+      <c r="F50" s="35"/>
+      <c r="G50" s="36"/>
+      <c r="H50" s="35"/>
+      <c r="I50" s="36"/>
+      <c r="J50" s="35"/>
+      <c r="K50" s="36"/>
+      <c r="L50" s="60"/>
+      <c r="M50" s="36"/>
+      <c r="N50" s="103" t="s">
+        <v>217</v>
+      </c>
+      <c r="O50" s="104"/>
+      <c r="P50" s="104"/>
+      <c r="Q50" s="56">
+        <f>SUM(Q10:Q49)</f>
+        <v>575.84830000000011</v>
+      </c>
+      <c r="R50" s="105"/>
+      <c r="S50" s="106"/>
     </row>
     <row r="51" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A51" s="1"/>
-      <c r="B51" s="32"/>
-      <c r="C51" s="43"/>
-      <c r="D51" s="33"/>
-      <c r="E51" s="34"/>
-      <c r="F51" s="35"/>
-      <c r="G51" s="36"/>
-      <c r="H51" s="35"/>
-      <c r="I51" s="36"/>
-      <c r="J51" s="35"/>
-      <c r="K51" s="36"/>
-      <c r="L51" s="60"/>
-      <c r="M51" s="36"/>
+      <c r="B51" s="25"/>
+      <c r="C51" s="44"/>
+      <c r="D51" s="9"/>
+      <c r="E51" s="10"/>
+      <c r="F51" s="10"/>
+      <c r="G51" s="10"/>
+      <c r="H51" s="10"/>
+      <c r="I51" s="10"/>
+      <c r="J51" s="10"/>
+      <c r="K51" s="10"/>
+      <c r="L51" s="10"/>
+      <c r="M51" s="10"/>
       <c r="N51" s="103" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="O51" s="104"/>
       <c r="P51" s="104"/>
-      <c r="Q51" s="56">
-        <f>SUM(Q10:Q50)</f>
-        <v>580.32130000000006</v>
-      </c>
-      <c r="R51" s="105"/>
-      <c r="S51" s="106"/>
-    </row>
-    <row r="52" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="1"/>
-      <c r="B52" s="25"/>
-      <c r="C52" s="44"/>
-      <c r="D52" s="9"/>
-      <c r="E52" s="10"/>
-      <c r="F52" s="10"/>
-      <c r="G52" s="10"/>
-      <c r="H52" s="10"/>
-      <c r="I52" s="10"/>
-      <c r="J52" s="10"/>
-      <c r="K52" s="10"/>
-      <c r="L52" s="10"/>
-      <c r="M52" s="10"/>
-      <c r="N52" s="103" t="s">
-        <v>218</v>
-      </c>
-      <c r="O52" s="104"/>
-      <c r="P52" s="104"/>
-      <c r="Q52" s="57">
-        <f>Q51/5</f>
-        <v>116.06426000000002</v>
-      </c>
-      <c r="R52" s="107"/>
-      <c r="S52" s="108"/>
+      <c r="Q51" s="57">
+        <f>Q50/5</f>
+        <v>115.16966000000002</v>
+      </c>
+      <c r="R51" s="107"/>
+      <c r="S51" s="108"/>
     </row>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="K1:S1"/>
     <mergeCell ref="S3:S8"/>
+    <mergeCell ref="N50:P50"/>
+    <mergeCell ref="R50:S51"/>
     <mergeCell ref="N51:P51"/>
-    <mergeCell ref="R51:S52"/>
-    <mergeCell ref="N52:P52"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="O14" r:id="rId1" xr:uid="{420DCDE1-6A77-47F4-86D9-3A6544D49E88}"/>
-    <hyperlink ref="O24" r:id="rId2" xr:uid="{AEB6D0A9-124F-4BCC-BD29-0DA5FC3E1114}"/>
-    <hyperlink ref="O25" r:id="rId3" xr:uid="{75B9793B-FDE1-4887-A636-2D7648FE5B59}"/>
-    <hyperlink ref="O27" r:id="rId4" xr:uid="{8B764C3B-B8EF-4167-AB42-B04A43058B58}"/>
-    <hyperlink ref="O30" r:id="rId5" xr:uid="{337B7D6D-9EB5-4E9C-99F9-0DD2C162AB67}"/>
-    <hyperlink ref="O45" r:id="rId6" xr:uid="{D3ABA29E-C6F5-40D5-9271-A39E1BA068DB}"/>
-    <hyperlink ref="O32" r:id="rId7" xr:uid="{1CC0740B-4EB1-4CC1-85F1-43A4CEF5DC65}"/>
-    <hyperlink ref="O41" r:id="rId8" xr:uid="{CAE463F4-1476-4F54-93B4-D67CA8F283F4}"/>
-    <hyperlink ref="O36" r:id="rId9" xr:uid="{92B089EB-AA8C-4C27-8523-6B1D8A81A23B}"/>
+    <hyperlink ref="O13" r:id="rId1" xr:uid="{420DCDE1-6A77-47F4-86D9-3A6544D49E88}"/>
+    <hyperlink ref="O22" r:id="rId2" xr:uid="{AEB6D0A9-124F-4BCC-BD29-0DA5FC3E1114}"/>
+    <hyperlink ref="O23" r:id="rId3" xr:uid="{75B9793B-FDE1-4887-A636-2D7648FE5B59}"/>
+    <hyperlink ref="O26" r:id="rId4" xr:uid="{8B764C3B-B8EF-4167-AB42-B04A43058B58}"/>
+    <hyperlink ref="O29" r:id="rId5" xr:uid="{337B7D6D-9EB5-4E9C-99F9-0DD2C162AB67}"/>
+    <hyperlink ref="O44" r:id="rId6" xr:uid="{D3ABA29E-C6F5-40D5-9271-A39E1BA068DB}"/>
+    <hyperlink ref="O31" r:id="rId7" xr:uid="{1CC0740B-4EB1-4CC1-85F1-43A4CEF5DC65}"/>
+    <hyperlink ref="O40" r:id="rId8" xr:uid="{CAE463F4-1476-4F54-93B4-D67CA8F283F4}"/>
+    <hyperlink ref="O35" r:id="rId9" xr:uid="{92B089EB-AA8C-4C27-8523-6B1D8A81A23B}"/>
     <hyperlink ref="O10" r:id="rId10" xr:uid="{3F7CE80E-842A-437C-893B-FEB4182CB4E3}"/>
-    <hyperlink ref="O11" r:id="rId11" xr:uid="{9E7B7C6F-0A2E-4BCB-B35E-43B466BFDA5C}"/>
-    <hyperlink ref="O13" r:id="rId12" xr:uid="{C8CC9CA7-E92A-4BBD-A0BA-5552E9421E8B}"/>
-    <hyperlink ref="O16" r:id="rId13" xr:uid="{60ADA263-0EC7-4F8B-850D-CFEC1BEB250E}"/>
-    <hyperlink ref="O17" r:id="rId14" xr:uid="{D777C9CD-6E10-4509-97B1-7BAD3C929690}"/>
-    <hyperlink ref="O19" r:id="rId15" xr:uid="{1D337CBF-01D5-437B-B79A-CCE149CAB43B}"/>
-    <hyperlink ref="O12" r:id="rId16" xr:uid="{76A51466-FB67-4F83-972F-53D4D8CC40CB}"/>
-    <hyperlink ref="O20" r:id="rId17" xr:uid="{018B0414-39A5-4AAD-AA7D-E61B78527009}"/>
-    <hyperlink ref="O21" r:id="rId18" xr:uid="{85AD460B-7E8F-4533-84C8-49E79DFFA46F}"/>
-    <hyperlink ref="O22" r:id="rId19" xr:uid="{5936EBB3-D5EF-4BB1-8C34-4A1B869D76E0}"/>
-    <hyperlink ref="O23" r:id="rId20" xr:uid="{94935E71-5D6F-424D-AA36-F94FBA6FD350}"/>
-    <hyperlink ref="O26" r:id="rId21" xr:uid="{10D03C81-3D73-4466-AD8F-3FD074D169E1}"/>
-    <hyperlink ref="O33" r:id="rId22" xr:uid="{515FE09E-3C15-4AA6-AC28-FC6848AB4CF9}"/>
-    <hyperlink ref="O34" r:id="rId23" xr:uid="{F184C3EB-9B39-4522-A425-F5E6C8F2E2BA}"/>
-    <hyperlink ref="O35" r:id="rId24" xr:uid="{7522B420-E61D-4B13-A03E-5D2219252C19}"/>
-    <hyperlink ref="O37" r:id="rId25" xr:uid="{1FAE88F3-D29C-4196-9AA0-EC0A26F8A675}"/>
-    <hyperlink ref="O38" r:id="rId26" xr:uid="{58C63D22-D4C4-4CC6-9C17-41BAEC714A2B}"/>
-    <hyperlink ref="O42" r:id="rId27" xr:uid="{FCE98D2C-0CE3-4786-B922-305B918F7C62}"/>
-    <hyperlink ref="O43" r:id="rId28" xr:uid="{849FD330-0BAA-4388-A88F-0CB639BF150A}"/>
-    <hyperlink ref="O49" r:id="rId29" xr:uid="{2178B7AB-D5B6-4299-9DFB-A14ABFBC6872}"/>
-    <hyperlink ref="O50" r:id="rId30" xr:uid="{941D925C-D957-48A4-B614-74212814F841}"/>
-    <hyperlink ref="O15" r:id="rId31" xr:uid="{22EC1134-DF98-4938-8100-CAD056F7A6FC}"/>
-    <hyperlink ref="O18" r:id="rId32" xr:uid="{27EEC157-09A7-49ED-9980-E1E26806C989}"/>
-    <hyperlink ref="O40" r:id="rId33" xr:uid="{AE8A45B1-317C-4A4A-B10C-C532A22ED538}"/>
-    <hyperlink ref="O46" r:id="rId34" xr:uid="{DF599000-74F0-4992-8A33-6279DB7AA224}"/>
-    <hyperlink ref="O28" r:id="rId35" xr:uid="{49460E9B-A839-49B1-A25F-76DFEA3F3059}"/>
+    <hyperlink ref="O12" r:id="rId11" xr:uid="{C8CC9CA7-E92A-4BBD-A0BA-5552E9421E8B}"/>
+    <hyperlink ref="O15" r:id="rId12" xr:uid="{60ADA263-0EC7-4F8B-850D-CFEC1BEB250E}"/>
+    <hyperlink ref="O16" r:id="rId13" xr:uid="{D777C9CD-6E10-4509-97B1-7BAD3C929690}"/>
+    <hyperlink ref="O19" r:id="rId14" xr:uid="{1D337CBF-01D5-437B-B79A-CCE149CAB43B}"/>
+    <hyperlink ref="O11" r:id="rId15" xr:uid="{76A51466-FB67-4F83-972F-53D4D8CC40CB}"/>
+    <hyperlink ref="O20" r:id="rId16" xr:uid="{018B0414-39A5-4AAD-AA7D-E61B78527009}"/>
+    <hyperlink ref="O17" r:id="rId17" xr:uid="{5936EBB3-D5EF-4BB1-8C34-4A1B869D76E0}"/>
+    <hyperlink ref="O25" r:id="rId18" xr:uid="{10D03C81-3D73-4466-AD8F-3FD074D169E1}"/>
+    <hyperlink ref="O32" r:id="rId19" xr:uid="{515FE09E-3C15-4AA6-AC28-FC6848AB4CF9}"/>
+    <hyperlink ref="O33" r:id="rId20" xr:uid="{F184C3EB-9B39-4522-A425-F5E6C8F2E2BA}"/>
+    <hyperlink ref="O34" r:id="rId21" xr:uid="{7522B420-E61D-4B13-A03E-5D2219252C19}"/>
+    <hyperlink ref="O36" r:id="rId22" xr:uid="{1FAE88F3-D29C-4196-9AA0-EC0A26F8A675}"/>
+    <hyperlink ref="O37" r:id="rId23" xr:uid="{58C63D22-D4C4-4CC6-9C17-41BAEC714A2B}"/>
+    <hyperlink ref="O41" r:id="rId24" xr:uid="{FCE98D2C-0CE3-4786-B922-305B918F7C62}"/>
+    <hyperlink ref="O42" r:id="rId25" xr:uid="{849FD330-0BAA-4388-A88F-0CB639BF150A}"/>
+    <hyperlink ref="O48" r:id="rId26" xr:uid="{2178B7AB-D5B6-4299-9DFB-A14ABFBC6872}"/>
+    <hyperlink ref="O49" r:id="rId27" xr:uid="{941D925C-D957-48A4-B614-74212814F841}"/>
+    <hyperlink ref="O14" r:id="rId28" xr:uid="{22EC1134-DF98-4938-8100-CAD056F7A6FC}"/>
+    <hyperlink ref="O18" r:id="rId29" xr:uid="{27EEC157-09A7-49ED-9980-E1E26806C989}"/>
+    <hyperlink ref="O39" r:id="rId30" xr:uid="{AE8A45B1-317C-4A4A-B10C-C532A22ED538}"/>
+    <hyperlink ref="O45" r:id="rId31" xr:uid="{DF599000-74F0-4992-8A33-6279DB7AA224}"/>
+    <hyperlink ref="O27" r:id="rId32" xr:uid="{49460E9B-A839-49B1-A25F-76DFEA3F3059}"/>
+    <hyperlink ref="O21" r:id="rId33" xr:uid="{85AD460B-7E8F-4533-84C8-49E79DFFA46F}"/>
+    <hyperlink ref="O24" r:id="rId34" xr:uid="{0B162636-2BBC-4A06-BD90-D02B36D1E21F}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId36"/>
+  <drawing r:id="rId35"/>
 </worksheet>
 </file>
 

</xml_diff>